<commit_message>
Kontrat verisi guncellendi: 2026-07-30
</commit_message>
<xml_diff>
--- a/marketpano.xlsx
+++ b/marketpano.xlsx
@@ -25456,13 +25456,13 @@
         </is>
       </c>
       <c r="O3" s="8" t="n">
-        <v>64066.4</v>
+        <v>64580.1</v>
       </c>
       <c r="P3" s="42" t="n">
         <v>0.0001</v>
       </c>
       <c r="Q3" s="43" t="n">
-        <v>6.40664</v>
+        <v>6.45801</v>
       </c>
       <c r="R3" s="42" t="n">
         <v>0.1</v>
@@ -25477,16 +25477,16 @@
         <v>100</v>
       </c>
       <c r="V3" s="46" t="n">
-        <v>0.00959333578841</v>
+        <v>0.00801821241469</v>
       </c>
       <c r="W3" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X3" s="9" t="n">
-        <v>2633873.09846</v>
+        <v>4286271.339899999</v>
       </c>
       <c r="Y3" s="46" t="n">
-        <v>0.0001560880586368905</v>
+        <v>0.0001548464619883599</v>
       </c>
       <c r="Z3" s="6" t="inlineStr">
         <is>
@@ -25528,7 +25528,7 @@
       </c>
       <c r="AL3" s="10" t="inlineStr"/>
       <c r="AM3" s="16" t="n">
-        <v>0</v>
+        <v>64598.1655</v>
       </c>
       <c r="AN3" s="54" t="n">
         <v>0.0001</v>
@@ -25549,24 +25549,26 @@
         <v>150</v>
       </c>
       <c r="AT3" s="58" t="n">
-        <v>0.007399999999999999</v>
+        <v>0.0041</v>
       </c>
       <c r="AU3" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV3" s="17" t="n">
-        <v>1683446.38004</v>
-      </c>
-      <c r="AW3" s="58" t="n"/>
+        <v>3829340.578670001</v>
+      </c>
+      <c r="AW3" s="58" t="n">
+        <v>0.000154883396033041</v>
+      </c>
       <c r="AX3" s="14" t="inlineStr"/>
       <c r="AY3" s="20" t="n">
-        <v>64175.52</v>
+        <v>64602.72</v>
       </c>
       <c r="AZ3" s="60" t="n">
         <v>0.0001</v>
       </c>
       <c r="BA3" s="61" t="n">
-        <v>6.414978000000001</v>
+        <v>6.457385</v>
       </c>
       <c r="BB3" s="60" t="n">
         <v>0.1</v>
@@ -25581,16 +25583,16 @@
         <v>200</v>
       </c>
       <c r="BF3" s="64" t="n">
-        <v>0.006200000000000001</v>
+        <v>0.0075</v>
       </c>
       <c r="BG3" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH3" s="21" t="n">
-        <v>2579979.701209999</v>
+        <v>2761444.29004</v>
       </c>
       <c r="BI3" s="64" t="n">
-        <v>0.0001558851799624953</v>
+        <v>0.0001548614493418323</v>
       </c>
       <c r="BJ3" s="18" t="inlineStr">
         <is>
@@ -25598,13 +25600,13 @@
         </is>
       </c>
       <c r="BK3" s="24" t="n">
-        <v>64194</v>
+        <v>64598.4</v>
       </c>
       <c r="BL3" s="66" t="n">
         <v>1e-05</v>
       </c>
       <c r="BM3" s="67" t="n">
-        <v>0.6417</v>
+        <v>0.64568</v>
       </c>
       <c r="BN3" s="66" t="n"/>
       <c r="BO3" s="68" t="n"/>
@@ -25615,16 +25617,16 @@
         <v>40</v>
       </c>
       <c r="BR3" s="70" t="n">
-        <v>0.00094944</v>
+        <v>0.0004740499999999999</v>
       </c>
       <c r="BS3" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT3" s="25" t="n">
-        <v>9067990.142309999</v>
+        <v>13277377.93493</v>
       </c>
       <c r="BU3" s="70" t="n">
-        <v>0.001558360604643915</v>
+        <v>0.001548754801139884</v>
       </c>
       <c r="BV3" s="22" t="inlineStr">
         <is>
@@ -25680,13 +25682,13 @@
         </is>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1905.7</v>
+        <v>1917.8</v>
       </c>
       <c r="P4" s="42" t="n">
         <v>0.001</v>
       </c>
       <c r="Q4" s="43" t="n">
-        <v>1.9057</v>
+        <v>1.9178</v>
       </c>
       <c r="R4" s="42" t="n">
         <v>0.01</v>
@@ -25701,16 +25703,16 @@
         <v>100</v>
       </c>
       <c r="V4" s="46" t="n">
-        <v>0.00228028757371</v>
+        <v>0.0004340339487</v>
       </c>
       <c r="W4" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X4" s="9" t="n">
-        <v>5684883.58086</v>
+        <v>6135804.530410001</v>
       </c>
       <c r="Y4" s="46" t="n">
-        <v>0.0005247415647788689</v>
+        <v>0.0005214308061315521</v>
       </c>
       <c r="Z4" s="6" t="inlineStr">
         <is>
@@ -25752,7 +25754,7 @@
       </c>
       <c r="AL4" s="10" t="inlineStr"/>
       <c r="AM4" s="16" t="n">
-        <v>0</v>
+        <v>1918.495</v>
       </c>
       <c r="AN4" s="54" t="n">
         <v>0.01</v>
@@ -25773,24 +25775,26 @@
         <v>150</v>
       </c>
       <c r="AT4" s="58" t="n">
-        <v>0.0051</v>
+        <v>0.0056</v>
       </c>
       <c r="AU4" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV4" s="17" t="n">
-        <v>2890003.0525</v>
-      </c>
-      <c r="AW4" s="58" t="n"/>
+        <v>6235724.150200002</v>
+      </c>
+      <c r="AW4" s="58" t="n">
+        <v>0.0005214933483518675</v>
+      </c>
       <c r="AX4" s="14" t="inlineStr"/>
       <c r="AY4" s="20" t="n">
-        <v>1909.53</v>
+        <v>1918.6</v>
       </c>
       <c r="AZ4" s="60" t="n">
         <v>0.01</v>
       </c>
       <c r="BA4" s="61" t="n">
-        <v>19.0866</v>
+        <v>19.177</v>
       </c>
       <c r="BB4" s="60" t="n">
         <v>0.01</v>
@@ -25805,16 +25809,16 @@
         <v>200</v>
       </c>
       <c r="BF4" s="64" t="n">
-        <v>-0.0019</v>
+        <v>0.0037</v>
       </c>
       <c r="BG4" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH4" s="21" t="n">
-        <v>1608011.2028</v>
+        <v>4123940.5376</v>
       </c>
       <c r="BI4" s="64" t="n">
-        <v>0.000523927781794081</v>
+        <v>0.0005214579965579029</v>
       </c>
       <c r="BJ4" s="18" t="inlineStr">
         <is>
@@ -25822,13 +25826,13 @@
         </is>
       </c>
       <c r="BK4" s="24" t="n">
-        <v>1909.6</v>
+        <v>1918.5</v>
       </c>
       <c r="BL4" s="66" t="n">
         <v>0.0001</v>
       </c>
       <c r="BM4" s="67" t="n">
-        <v>0.19089</v>
+        <v>0.19177</v>
       </c>
       <c r="BN4" s="66" t="n"/>
       <c r="BO4" s="68" t="n"/>
@@ -25839,16 +25843,16 @@
         <v>25</v>
       </c>
       <c r="BR4" s="70" t="n">
-        <v>0.00121841</v>
+        <v>0.0007186499999999999</v>
       </c>
       <c r="BS4" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT4" s="25" t="n">
-        <v>24119096.15741</v>
+        <v>26403743.56615001</v>
       </c>
       <c r="BU4" s="70" t="n">
-        <v>0.005238619100000474</v>
+        <v>0.005214579965590886</v>
       </c>
       <c r="BV4" s="22" t="inlineStr">
         <is>
@@ -25988,13 +25992,13 @@
         </is>
       </c>
       <c r="O6" s="8" t="n">
-        <v>575.5</v>
+        <v>580.7</v>
       </c>
       <c r="P6" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q6" s="43" t="n">
-        <v>5.755</v>
+        <v>5.807</v>
       </c>
       <c r="R6" s="42" t="n">
         <v>0.1</v>
@@ -26015,10 +26019,10 @@
         <v>8</v>
       </c>
       <c r="X6" s="9" t="n">
-        <v>9194319.189999998</v>
+        <v>9719733.256999999</v>
       </c>
       <c r="Y6" s="46" t="n">
-        <v>0.01737619461338362</v>
+        <v>0.01722059583260015</v>
       </c>
       <c r="Z6" s="6" t="inlineStr">
         <is>
@@ -26060,7 +26064,7 @@
       </c>
       <c r="AL6" s="10" t="inlineStr"/>
       <c r="AM6" s="16" t="n">
-        <v>0</v>
+        <v>581.0717176455673</v>
       </c>
       <c r="AN6" s="54" t="n">
         <v>0.01</v>
@@ -26087,18 +26091,20 @@
         <v>8</v>
       </c>
       <c r="AV6" s="17" t="n">
-        <v>732279.6496999998</v>
-      </c>
-      <c r="AW6" s="58" t="n"/>
+        <v>1136383.4495</v>
+      </c>
+      <c r="AW6" s="58" t="n">
+        <v>0.001722326518659841</v>
+      </c>
       <c r="AX6" s="14" t="inlineStr"/>
       <c r="AY6" s="20" t="n">
-        <v>576.115</v>
+        <v>581.0700000000001</v>
       </c>
       <c r="AZ6" s="60" t="n">
         <v>0.001</v>
       </c>
       <c r="BA6" s="61" t="n">
-        <v>0.5759</v>
+        <v>0.5808</v>
       </c>
       <c r="BB6" s="60" t="n">
         <v>0.05</v>
@@ -26113,16 +26119,16 @@
         <v>75</v>
       </c>
       <c r="BF6" s="64" t="n">
-        <v>-0.0038</v>
+        <v>0.006200000000000001</v>
       </c>
       <c r="BG6" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH6" s="21" t="n">
-        <v>1975367.55665</v>
+        <v>1991466.51635</v>
       </c>
       <c r="BI6" s="64" t="n">
-        <v>0.008682062858146938</v>
+        <v>0.008608815426989417</v>
       </c>
       <c r="BJ6" s="18" t="inlineStr">
         <is>
@@ -26130,13 +26136,13 @@
         </is>
       </c>
       <c r="BK6" s="24" t="n">
-        <v>576.29</v>
+        <v>581.05</v>
       </c>
       <c r="BL6" s="66" t="n">
         <v>0.001</v>
       </c>
       <c r="BM6" s="67" t="n">
-        <v>0.57621</v>
+        <v>0.58108</v>
       </c>
       <c r="BN6" s="66" t="n"/>
       <c r="BO6" s="68" t="n"/>
@@ -26153,10 +26159,10 @@
         <v>1</v>
       </c>
       <c r="BT6" s="25" t="n">
-        <v>209068.80274</v>
+        <v>202788.71276</v>
       </c>
       <c r="BU6" s="70" t="n">
-        <v>0.001735478384615141</v>
+        <v>0.001720933434293196</v>
       </c>
       <c r="BV6" s="22" t="inlineStr">
         <is>
@@ -26212,13 +26218,13 @@
         </is>
       </c>
       <c r="O7" s="8" t="n">
-        <v>1.001206</v>
+        <v>1.000908</v>
       </c>
       <c r="P7" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q7" s="43" t="n">
-        <v>10.01206</v>
+        <v>10.00908</v>
       </c>
       <c r="R7" s="42" t="n">
         <v>1e-06</v>
@@ -26239,10 +26245,10 @@
         <v>8</v>
       </c>
       <c r="X7" s="9" t="n">
-        <v>179712.11746</v>
+        <v>253509.9992</v>
       </c>
       <c r="Y7" s="46" t="n">
-        <v>9.987954528236726e-05</v>
+        <v>0.002797459906418874</v>
       </c>
       <c r="Z7" s="6" t="inlineStr">
         <is>
@@ -26262,7 +26268,7 @@
       <c r="AK7" s="52" t="n"/>
       <c r="AL7" s="10" t="inlineStr"/>
       <c r="AM7" s="16" t="n">
-        <v>0</v>
+        <v>1.001162289806309</v>
       </c>
       <c r="AN7" s="54" t="n">
         <v>0.1</v>
@@ -26283,18 +26289,20 @@
         <v>50</v>
       </c>
       <c r="AT7" s="58" t="n">
-        <v>-0.0012</v>
+        <v>0.001</v>
       </c>
       <c r="AU7" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV7" s="17" t="n">
-        <v>1194750.53657</v>
-      </c>
-      <c r="AW7" s="58" t="n"/>
+        <v>3189278.13574</v>
+      </c>
+      <c r="AW7" s="58" t="n">
+        <v>0.0299790146897139</v>
+      </c>
       <c r="AX7" s="14" t="inlineStr"/>
       <c r="AY7" s="20" t="n">
-        <v>1.00115</v>
+        <v>1.00117</v>
       </c>
       <c r="AZ7" s="60" t="n">
         <v>1</v>
@@ -26315,16 +26323,16 @@
         <v>50</v>
       </c>
       <c r="BF7" s="64" t="n">
-        <v>0.0036</v>
+        <v>0.0007999999999999999</v>
       </c>
       <c r="BG7" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH7" s="21" t="n">
-        <v>62125.29829999998</v>
+        <v>61772.41849999997</v>
       </c>
       <c r="BI7" s="64" t="n">
-        <v>0.09999999999998899</v>
+        <v>0.08999999999999009</v>
       </c>
       <c r="BJ7" s="18" t="inlineStr">
         <is>
@@ -26392,13 +26400,13 @@
         </is>
       </c>
       <c r="O8" s="8" t="n">
-        <v>1.0764</v>
+        <v>1.0811</v>
       </c>
       <c r="P8" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q8" s="43" t="n">
-        <v>1.0764</v>
+        <v>1.0811</v>
       </c>
       <c r="R8" s="42" t="n">
         <v>0.0001</v>
@@ -26413,16 +26421,16 @@
         <v>100</v>
       </c>
       <c r="V8" s="46" t="n">
-        <v>0.00602271308437</v>
+        <v>0.00354304590723</v>
       </c>
       <c r="W8" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X8" s="9" t="n">
-        <v>9059653.606900001</v>
+        <v>9647178.890299998</v>
       </c>
       <c r="Y8" s="46" t="n">
-        <v>0.009290226681530006</v>
+        <v>0.009249838127831745</v>
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
@@ -26442,7 +26450,7 @@
       <c r="AK8" s="52" t="n"/>
       <c r="AL8" s="10" t="inlineStr"/>
       <c r="AM8" s="16" t="n">
-        <v>0</v>
+        <v>1.081278700357021</v>
       </c>
       <c r="AN8" s="54" t="n">
         <v>1</v>
@@ -26463,24 +26471,26 @@
         <v>125</v>
       </c>
       <c r="AT8" s="58" t="n">
-        <v>0.007899999999999999</v>
+        <v>0.0072</v>
       </c>
       <c r="AU8" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV8" s="17" t="n">
-        <v>8029256.766200001</v>
-      </c>
-      <c r="AW8" s="58" t="n"/>
+        <v>14418308.214</v>
+      </c>
+      <c r="AW8" s="58" t="n">
+        <v>0.009252405625461603</v>
+      </c>
       <c r="AX8" s="14" t="inlineStr"/>
       <c r="AY8" s="20" t="n">
-        <v>1.0779</v>
+        <v>1.0817</v>
       </c>
       <c r="AZ8" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA8" s="61" t="n">
-        <v>10.778</v>
+        <v>10.811</v>
       </c>
       <c r="BB8" s="60" t="n">
         <v>0.0001</v>
@@ -26495,16 +26505,16 @@
         <v>100</v>
       </c>
       <c r="BF8" s="64" t="n">
-        <v>0.0009</v>
+        <v>-0.004</v>
       </c>
       <c r="BG8" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH8" s="21" t="n">
-        <v>1993353.966999999</v>
+        <v>2130338.992999999</v>
       </c>
       <c r="BI8" s="64" t="n">
-        <v>0.009278159213231678</v>
+        <v>0.009249838127831745</v>
       </c>
       <c r="BJ8" s="18" t="inlineStr">
         <is>
@@ -26512,13 +26522,13 @@
         </is>
       </c>
       <c r="BK8" s="24" t="n">
-        <v>1.078303</v>
+        <v>1.081222</v>
       </c>
       <c r="BL8" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM8" s="67" t="n">
-        <v>1.0778</v>
+        <v>1.0808</v>
       </c>
       <c r="BN8" s="66" t="n"/>
       <c r="BO8" s="68" t="n"/>
@@ -26535,10 +26545,10 @@
         <v>1</v>
       </c>
       <c r="BT8" s="25" t="n">
-        <v>3889871.182699999</v>
+        <v>3675929.733</v>
       </c>
       <c r="BU8" s="70" t="n">
-        <v>0.009278159213211077</v>
+        <v>0.009252405625461603</v>
       </c>
       <c r="BV8" s="22" t="inlineStr">
         <is>
@@ -26594,13 +26604,13 @@
         </is>
       </c>
       <c r="O9" s="8" t="n">
-        <v>73.31999999999999</v>
+        <v>73.97</v>
       </c>
       <c r="P9" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q9" s="43" t="n">
-        <v>0.7332</v>
+        <v>0.7397</v>
       </c>
       <c r="R9" s="42" t="n">
         <v>0.01</v>
@@ -26615,16 +26625,16 @@
         <v>100</v>
       </c>
       <c r="V9" s="46" t="n">
-        <v>0.00031710995296</v>
+        <v>-0.00476698164898</v>
       </c>
       <c r="W9" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X9" s="9" t="n">
-        <v>17897617.3257</v>
+        <v>22763458.7548</v>
       </c>
       <c r="Y9" s="46" t="n">
-        <v>0.01363884342608445</v>
+        <v>0.01351899418683942</v>
       </c>
       <c r="Z9" s="6" t="inlineStr">
         <is>
@@ -26644,7 +26654,7 @@
       <c r="AK9" s="52" t="n"/>
       <c r="AL9" s="10" t="inlineStr"/>
       <c r="AM9" s="16" t="n">
-        <v>0</v>
+        <v>74.1075</v>
       </c>
       <c r="AN9" s="54" t="n">
         <v>0.1</v>
@@ -26665,24 +26675,26 @@
         <v>100</v>
       </c>
       <c r="AT9" s="58" t="n">
-        <v>0.0029</v>
+        <v>0.0034</v>
       </c>
       <c r="AU9" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV9" s="17" t="n">
-        <v>1705160.1391</v>
-      </c>
-      <c r="AW9" s="58" t="n"/>
+        <v>4517871.882900001</v>
+      </c>
+      <c r="AW9" s="58" t="n">
+        <v>0.001350128937300774</v>
+      </c>
       <c r="AX9" s="14" t="inlineStr"/>
       <c r="AY9" s="20" t="n">
-        <v>73.53400000000001</v>
+        <v>74.12</v>
       </c>
       <c r="AZ9" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA9" s="61" t="n">
-        <v>73.52</v>
+        <v>74.08</v>
       </c>
       <c r="BB9" s="60" t="n">
         <v>0.01</v>
@@ -26697,16 +26709,16 @@
         <v>100</v>
       </c>
       <c r="BF9" s="64" t="n">
-        <v>0.0029</v>
+        <v>-0.0026</v>
       </c>
       <c r="BG9" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH9" s="21" t="n">
-        <v>4686389.819999999</v>
+        <v>6082881.439999999</v>
       </c>
       <c r="BI9" s="64" t="n">
-        <v>0.01360174102285788</v>
+        <v>0.01349892008638081</v>
       </c>
       <c r="BJ9" s="18" t="inlineStr">
         <is>
@@ -26714,13 +26726,13 @@
         </is>
       </c>
       <c r="BK9" s="24" t="n">
-        <v>73.58499999999999</v>
+        <v>74.1066</v>
       </c>
       <c r="BL9" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM9" s="67" t="n">
-        <v>0.7354900000000001</v>
+        <v>0.7406900000000001</v>
       </c>
       <c r="BN9" s="66" t="n"/>
       <c r="BO9" s="68" t="n"/>
@@ -26731,16 +26743,16 @@
         <v>20</v>
       </c>
       <c r="BR9" s="70" t="n">
-        <v>0.00125</v>
+        <v>0.00012995</v>
       </c>
       <c r="BS9" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT9" s="25" t="n">
-        <v>1584659.26468</v>
+        <v>1332725.76888</v>
       </c>
       <c r="BU9" s="70" t="n">
-        <v>0.001359637792498572</v>
+        <v>0.001350092481322232</v>
       </c>
       <c r="BV9" s="22" t="inlineStr">
         <is>
@@ -26796,13 +26808,13 @@
         </is>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0.32779</v>
+        <v>0.32846</v>
       </c>
       <c r="P10" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q10" s="43" t="n">
-        <v>3.2779</v>
+        <v>3.2846</v>
       </c>
       <c r="R10" s="42" t="n">
         <v>1e-05</v>
@@ -26817,16 +26829,16 @@
         <v>50</v>
       </c>
       <c r="V10" s="46" t="n">
-        <v>-0.0026051918292</v>
+        <v>0.00398924372231</v>
       </c>
       <c r="W10" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X10" s="9" t="n">
-        <v>561059.6984000002</v>
+        <v>522089.0857000002</v>
       </c>
       <c r="Y10" s="46" t="n">
-        <v>0.003050733701458251</v>
+        <v>0.003044510747109082</v>
       </c>
       <c r="Z10" s="6" t="inlineStr">
         <is>
@@ -26846,7 +26858,7 @@
       <c r="AK10" s="52" t="n"/>
       <c r="AL10" s="10" t="inlineStr"/>
       <c r="AM10" s="16" t="n">
-        <v>0</v>
+        <v>0.3286052053374287</v>
       </c>
       <c r="AN10" s="54" t="n">
         <v>1</v>
@@ -26867,24 +26879,26 @@
         <v>75</v>
       </c>
       <c r="AT10" s="58" t="n">
-        <v>0.007399999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="AU10" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV10" s="17" t="n">
-        <v>313835.65166</v>
-      </c>
-      <c r="AW10" s="58" t="n"/>
+        <v>687724.7170799999</v>
+      </c>
+      <c r="AW10" s="58" t="n">
+        <v>0.003045066991476858</v>
+      </c>
       <c r="AX10" s="14" t="inlineStr"/>
       <c r="AY10" s="20" t="n">
-        <v>0.327986</v>
+        <v>0.32861</v>
       </c>
       <c r="AZ10" s="60" t="n">
         <v>100</v>
       </c>
       <c r="BA10" s="61" t="n">
-        <v>32.774</v>
+        <v>32.844</v>
       </c>
       <c r="BB10" s="60" t="n">
         <v>1e-05</v>
@@ -26899,16 +26913,16 @@
         <v>75</v>
       </c>
       <c r="BF10" s="64" t="n">
-        <v>0.0027</v>
+        <v>0.0042</v>
       </c>
       <c r="BG10" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH10" s="21" t="n">
-        <v>147027.128</v>
+        <v>136706.7439999999</v>
       </c>
       <c r="BI10" s="64" t="n">
-        <v>0.003051199121240767</v>
+        <v>0.00304469613932834</v>
       </c>
       <c r="BJ10" s="18" t="inlineStr">
         <is>
@@ -26916,13 +26930,13 @@
         </is>
       </c>
       <c r="BK10" s="24" t="n">
-        <v>0.327991</v>
+        <v>0.3286</v>
       </c>
       <c r="BL10" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM10" s="67" t="n">
-        <v>0.3278</v>
+        <v>0.32845</v>
       </c>
       <c r="BN10" s="66" t="n"/>
       <c r="BO10" s="68" t="n"/>
@@ -26939,10 +26953,10 @@
         <v>1</v>
       </c>
       <c r="BT10" s="25" t="n">
-        <v>110282.49038</v>
+        <v>98349.42459000001</v>
       </c>
       <c r="BU10" s="70" t="n">
-        <v>0.006101281269055672</v>
+        <v>0.003044603440388031</v>
       </c>
       <c r="BV10" s="22" t="inlineStr">
         <is>
@@ -26998,13 +27012,13 @@
         </is>
       </c>
       <c r="O11" s="8" t="n">
-        <v>53.783</v>
+        <v>53.973</v>
       </c>
       <c r="P11" s="42" t="n">
         <v>0.1</v>
       </c>
       <c r="Q11" s="43" t="n">
-        <v>5.3783</v>
+        <v>5.3973</v>
       </c>
       <c r="R11" s="42" t="n">
         <v>0.001</v>
@@ -27019,16 +27033,16 @@
         <v>50</v>
       </c>
       <c r="V11" s="46" t="n">
-        <v>0.00234479334389</v>
+        <v>0.009143459865009999</v>
       </c>
       <c r="W11" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X11" s="9" t="n">
-        <v>389472.7661000001</v>
+        <v>426235.1671000001</v>
       </c>
       <c r="Y11" s="46" t="n">
-        <v>0.00185932357807796</v>
+        <v>0.00185277824096802</v>
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
@@ -27070,7 +27084,7 @@
       </c>
       <c r="AL11" s="10" t="inlineStr"/>
       <c r="AM11" s="16" t="n">
-        <v>0</v>
+        <v>54.1208200838145</v>
       </c>
       <c r="AN11" s="54" t="n">
         <v>0.01</v>
@@ -27091,24 +27105,26 @@
         <v>75</v>
       </c>
       <c r="AT11" s="58" t="n">
-        <v>-0.0015</v>
+        <v>0.0007999999999999999</v>
       </c>
       <c r="AU11" s="59" t="n">
         <v>4</v>
       </c>
       <c r="AV11" s="17" t="n">
-        <v>243786.30158</v>
-      </c>
-      <c r="AW11" s="58" t="n"/>
+        <v>541094.6764000001</v>
+      </c>
+      <c r="AW11" s="58" t="n">
+        <v>0.005546209166035225</v>
+      </c>
       <c r="AX11" s="14" t="inlineStr"/>
       <c r="AY11" s="20" t="n">
-        <v>53.982</v>
+        <v>54.099</v>
       </c>
       <c r="AZ11" s="60" t="n">
         <v>0.1</v>
       </c>
       <c r="BA11" s="61" t="n">
-        <v>5.3952</v>
+        <v>5.407500000000001</v>
       </c>
       <c r="BB11" s="60" t="n">
         <v>0.001</v>
@@ -27123,16 +27139,16 @@
         <v>75</v>
       </c>
       <c r="BF11" s="64" t="n">
-        <v>0.0042</v>
+        <v>0.0048</v>
       </c>
       <c r="BG11" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH11" s="21" t="n">
-        <v>159991.2424</v>
+        <v>166982.7439</v>
       </c>
       <c r="BI11" s="64" t="n">
-        <v>0.00185349940688904</v>
+        <v>0.001849283402690291</v>
       </c>
       <c r="BJ11" s="18" t="inlineStr">
         <is>
@@ -27140,13 +27156,13 @@
         </is>
       </c>
       <c r="BK11" s="24" t="n">
-        <v>53.9535</v>
+        <v>54.06</v>
       </c>
       <c r="BL11" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM11" s="67" t="n">
-        <v>0.539498</v>
+        <v>0.54039</v>
       </c>
       <c r="BN11" s="66" t="n"/>
       <c r="BO11" s="68" t="n"/>
@@ -27163,10 +27179,10 @@
         <v>1</v>
       </c>
       <c r="BT11" s="25" t="n">
-        <v>278135.69605</v>
+        <v>250543.6583</v>
       </c>
       <c r="BU11" s="70" t="n">
-        <v>0.001853574990079054</v>
+        <v>0.001850515368525823</v>
       </c>
       <c r="BV11" s="22" t="inlineStr">
         <is>
@@ -27222,13 +27238,13 @@
         </is>
       </c>
       <c r="O12" s="8" t="n">
-        <v>0.06977999999999999</v>
+        <v>0.07006999999999999</v>
       </c>
       <c r="P12" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q12" s="43" t="n">
-        <v>0.6978</v>
+        <v>0.7006999999999999</v>
       </c>
       <c r="R12" s="42" t="n">
         <v>1e-05</v>
@@ -27243,16 +27259,16 @@
         <v>50</v>
       </c>
       <c r="V12" s="46" t="n">
-        <v>0.00556049996757</v>
+        <v>0.00283107631055</v>
       </c>
       <c r="W12" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X12" s="9" t="n">
-        <v>14891574.2899</v>
+        <v>14411357.4165</v>
       </c>
       <c r="Y12" s="46" t="n">
-        <v>0.01433075379766409</v>
+        <v>0.01427144284288569</v>
       </c>
       <c r="Z12" s="6" t="inlineStr">
         <is>
@@ -27294,7 +27310,7 @@
       </c>
       <c r="AL12" s="10" t="inlineStr"/>
       <c r="AM12" s="16" t="n">
-        <v>0</v>
+        <v>0.07025746025146069</v>
       </c>
       <c r="AN12" s="54" t="n">
         <v>1</v>
@@ -27321,18 +27337,20 @@
         <v>8</v>
       </c>
       <c r="AV12" s="17" t="n">
-        <v>5401632.101999999</v>
-      </c>
-      <c r="AW12" s="58" t="n"/>
+        <v>11352587.71676</v>
+      </c>
+      <c r="AW12" s="58" t="n">
+        <v>0.01424095699230436</v>
+      </c>
       <c r="AX12" s="14" t="inlineStr"/>
       <c r="AY12" s="20" t="n">
-        <v>0.070008</v>
+        <v>0.07023799999999999</v>
       </c>
       <c r="AZ12" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA12" s="61" t="n">
-        <v>0.6997</v>
+        <v>0.702</v>
       </c>
       <c r="BB12" s="60" t="n">
         <v>1e-05</v>
@@ -27347,16 +27365,16 @@
         <v>75</v>
       </c>
       <c r="BF12" s="64" t="n">
-        <v>-0.0072</v>
+        <v>9.999999999999999e-05</v>
       </c>
       <c r="BG12" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH12" s="21" t="n">
-        <v>2310195.801099999</v>
+        <v>2415514.4953</v>
       </c>
       <c r="BI12" s="64" t="n">
-        <v>0.01429183935972006</v>
+        <v>0.01424501424500872</v>
       </c>
       <c r="BJ12" s="18" t="inlineStr">
         <is>
@@ -27364,13 +27382,13 @@
         </is>
       </c>
       <c r="BK12" s="24" t="n">
-        <v>0.070025</v>
+        <v>0.070255</v>
       </c>
       <c r="BL12" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM12" s="67" t="n">
-        <v>0.069982</v>
+        <v>0.070214</v>
       </c>
       <c r="BN12" s="66" t="n"/>
       <c r="BO12" s="68" t="n"/>
@@ -27381,16 +27399,16 @@
         <v>10</v>
       </c>
       <c r="BR12" s="70" t="n">
-        <v>-0.00077312</v>
+        <v>-4.763e-05</v>
       </c>
       <c r="BS12" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT12" s="25" t="n">
-        <v>266442.4860070001</v>
+        <v>383893.9257419999</v>
       </c>
       <c r="BU12" s="70" t="n">
-        <v>0.002857877739993141</v>
+        <v>0.001424217392544222</v>
       </c>
       <c r="BV12" s="22" t="inlineStr">
         <is>
@@ -27530,13 +27548,13 @@
         </is>
       </c>
       <c r="O14" s="8" t="n">
-        <v>475.14</v>
+        <v>476.95</v>
       </c>
       <c r="P14" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q14" s="43" t="n">
-        <v>4.7514</v>
+        <v>4.7695</v>
       </c>
       <c r="R14" s="42" t="n">
         <v>0.01</v>
@@ -27551,16 +27569,16 @@
         <v>50</v>
       </c>
       <c r="V14" s="46" t="n">
-        <v>-0.01016523048261</v>
+        <v>-0.005535061372419999</v>
       </c>
       <c r="W14" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X14" s="9" t="n">
-        <v>334898.4801</v>
+        <v>358296.3792</v>
       </c>
       <c r="Y14" s="46" t="n">
-        <v>0.00210464284210778</v>
+        <v>0.002096655833942951</v>
       </c>
       <c r="Z14" s="6" t="inlineStr">
         <is>
@@ -27580,7 +27598,7 @@
       <c r="AK14" s="52" t="n"/>
       <c r="AL14" s="10" t="inlineStr"/>
       <c r="AM14" s="16" t="n">
-        <v>0</v>
+        <v>477.2256745686288</v>
       </c>
       <c r="AN14" s="54" t="n">
         <v>0.001</v>
@@ -27601,24 +27619,26 @@
         <v>75</v>
       </c>
       <c r="AT14" s="58" t="n">
-        <v>-0.0272</v>
+        <v>-0.021</v>
       </c>
       <c r="AU14" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV14" s="17" t="n">
-        <v>129644.50743</v>
-      </c>
-      <c r="AW14" s="58" t="n"/>
+        <v>1027287.52802</v>
+      </c>
+      <c r="AW14" s="58" t="n">
+        <v>0.002097051545537002</v>
+      </c>
       <c r="AX14" s="14" t="inlineStr"/>
       <c r="AY14" s="20" t="n">
-        <v>475.883</v>
+        <v>477.25</v>
       </c>
       <c r="AZ14" s="60" t="n">
         <v>0.01</v>
       </c>
       <c r="BA14" s="61" t="n">
-        <v>4.755500000000001</v>
+        <v>4.769</v>
       </c>
       <c r="BB14" s="60" t="n">
         <v>0.01</v>
@@ -27633,16 +27653,16 @@
         <v>75</v>
       </c>
       <c r="BF14" s="64" t="n">
-        <v>-0.007600000000000001</v>
+        <v>-0.0124</v>
       </c>
       <c r="BG14" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH14" s="21" t="n">
-        <v>122255.3269</v>
+        <v>218448.6891</v>
       </c>
       <c r="BI14" s="64" t="n">
-        <v>0.00210282830406706</v>
+        <v>0.002096875655271735</v>
       </c>
       <c r="BJ14" s="18" t="inlineStr">
         <is>
@@ -27650,13 +27670,13 @@
         </is>
       </c>
       <c r="BK14" s="24" t="n">
-        <v>475.9225</v>
+        <v>476.95</v>
       </c>
       <c r="BL14" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM14" s="67" t="n">
-        <v>4.7577</v>
+        <v>4.768</v>
       </c>
       <c r="BN14" s="66" t="n"/>
       <c r="BO14" s="68" t="n"/>
@@ -27673,10 +27693,10 @@
         <v>1</v>
       </c>
       <c r="BT14" s="25" t="n">
-        <v>107827.0087</v>
+        <v>135389.3587</v>
       </c>
       <c r="BU14" s="70" t="n">
-        <v>0.006305567816388078</v>
+        <v>0.00629194630871911</v>
       </c>
       <c r="BV14" s="22" t="inlineStr">
         <is>
@@ -27756,7 +27776,7 @@
       <c r="AK15" s="52" t="n"/>
       <c r="AL15" s="10" t="inlineStr"/>
       <c r="AM15" s="16" t="n">
-        <v>0</v>
+        <v>357.3839958421593</v>
       </c>
       <c r="AN15" s="54" t="n">
         <v>0.01</v>
@@ -27783,18 +27803,20 @@
         <v>8</v>
       </c>
       <c r="AV15" s="17" t="n">
-        <v>244995.9703</v>
-      </c>
-      <c r="AW15" s="58" t="n"/>
+        <v>509031.192</v>
+      </c>
+      <c r="AW15" s="58" t="n">
+        <v>0.03636974037600589</v>
+      </c>
       <c r="AX15" s="14" t="inlineStr"/>
       <c r="AY15" s="20" t="n">
-        <v>354.923</v>
+        <v>357.43</v>
       </c>
       <c r="AZ15" s="60" t="n">
         <v>0.01</v>
       </c>
       <c r="BA15" s="61" t="n">
-        <v>3.5452</v>
+        <v>3.5745</v>
       </c>
       <c r="BB15" s="60" t="n">
         <v>0.01</v>
@@ -27815,10 +27837,10 @@
         <v>8</v>
       </c>
       <c r="BH15" s="21" t="n">
-        <v>146726.7861000001</v>
+        <v>194631.5569999999</v>
       </c>
       <c r="BI15" s="64" t="n">
-        <v>0.002820715333405987</v>
+        <v>0.07833263393480842</v>
       </c>
       <c r="BJ15" s="18" t="inlineStr">
         <is>
@@ -27826,13 +27848,13 @@
         </is>
       </c>
       <c r="BK15" s="24" t="n">
-        <v>354.42</v>
+        <v>357.68</v>
       </c>
       <c r="BL15" s="66" t="n">
         <v>0.001</v>
       </c>
       <c r="BM15" s="67" t="n">
-        <v>0.35431</v>
+        <v>0.35743</v>
       </c>
       <c r="BN15" s="66" t="n"/>
       <c r="BO15" s="68" t="n"/>
@@ -27849,10 +27871,10 @@
         <v>1</v>
       </c>
       <c r="BT15" s="25" t="n">
-        <v>68512.58916</v>
+        <v>73676.17165000002</v>
       </c>
       <c r="BU15" s="70" t="n">
-        <v>0.008467161525210327</v>
+        <v>0.01678650365106518</v>
       </c>
       <c r="BV15" s="22" t="inlineStr">
         <is>
@@ -27908,13 +27930,13 @@
         </is>
       </c>
       <c r="O16" s="8" t="n">
-        <v>8.300000000000001</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="P16" s="42" t="n">
         <v>0.1</v>
       </c>
       <c r="Q16" s="43" t="n">
-        <v>0.8300000000000001</v>
+        <v>0.837</v>
       </c>
       <c r="R16" s="42" t="n">
         <v>0.001</v>
@@ -27929,16 +27951,16 @@
         <v>50</v>
       </c>
       <c r="V16" s="46" t="n">
-        <v>0.00756200283755</v>
+        <v>0.006136734503550001</v>
       </c>
       <c r="W16" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X16" s="9" t="n">
-        <v>2660043.183899999</v>
+        <v>2776295.8839</v>
       </c>
       <c r="Y16" s="46" t="n">
-        <v>0.01204819277109906</v>
+        <v>0.01194743130228461</v>
       </c>
       <c r="Z16" s="6" t="inlineStr">
         <is>
@@ -27980,7 +28002,7 @@
       </c>
       <c r="AL16" s="10" t="inlineStr"/>
       <c r="AM16" s="16" t="n">
-        <v>0</v>
+        <v>8.370649913606998</v>
       </c>
       <c r="AN16" s="54" t="n">
         <v>1</v>
@@ -28001,24 +28023,26 @@
         <v>75</v>
       </c>
       <c r="AT16" s="58" t="n">
-        <v>0.006600000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="AU16" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV16" s="17" t="n">
-        <v>1866421.105</v>
-      </c>
-      <c r="AW16" s="58" t="n"/>
+        <v>4131154.858</v>
+      </c>
+      <c r="AW16" s="58" t="n">
+        <v>0.01195457262402207</v>
+      </c>
       <c r="AX16" s="14" t="inlineStr"/>
       <c r="AY16" s="20" t="n">
-        <v>8.3142</v>
+        <v>8.375299999999999</v>
       </c>
       <c r="AZ16" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA16" s="61" t="n">
-        <v>8.314</v>
+        <v>8.369</v>
       </c>
       <c r="BB16" s="60" t="n">
         <v>0.001</v>
@@ -28033,16 +28057,16 @@
         <v>75</v>
       </c>
       <c r="BF16" s="64" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0057</v>
       </c>
       <c r="BG16" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH16" s="21" t="n">
-        <v>1462301.135</v>
+        <v>1430493.682999999</v>
       </c>
       <c r="BI16" s="64" t="n">
-        <v>0.01202790473900917</v>
+        <v>0.01194885888396996</v>
       </c>
       <c r="BJ16" s="18" t="inlineStr">
         <is>
@@ -28050,13 +28074,13 @@
         </is>
       </c>
       <c r="BK16" s="24" t="n">
-        <v>8.3215</v>
+        <v>8.3705</v>
       </c>
       <c r="BL16" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM16" s="67" t="n">
-        <v>0.8316000000000001</v>
+        <v>0.8364800000000001</v>
       </c>
       <c r="BN16" s="66" t="n"/>
       <c r="BO16" s="68" t="n"/>
@@ -28067,16 +28091,16 @@
         <v>10</v>
       </c>
       <c r="BR16" s="70" t="n">
-        <v>0.00042423</v>
+        <v>0.00025076</v>
       </c>
       <c r="BS16" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT16" s="25" t="n">
-        <v>184254.39036</v>
+        <v>124309.01404</v>
       </c>
       <c r="BU16" s="70" t="n">
-        <v>0.0012025012024984</v>
+        <v>0.001195485845444804</v>
       </c>
       <c r="BV16" s="22" t="inlineStr">
         <is>
@@ -28132,13 +28156,13 @@
         </is>
       </c>
       <c r="O17" s="8" t="n">
-        <v>0.1636</v>
+        <v>0.1644</v>
       </c>
       <c r="P17" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q17" s="43" t="n">
-        <v>1.636</v>
+        <v>1.644</v>
       </c>
       <c r="R17" s="42" t="n">
         <v>0.0001</v>
@@ -28159,10 +28183,10 @@
         <v>8</v>
       </c>
       <c r="X17" s="9" t="n">
-        <v>1991932.14</v>
+        <v>2154138.162</v>
       </c>
       <c r="Y17" s="46" t="n">
-        <v>0.06112469437653835</v>
+        <v>0.06082725060826581</v>
       </c>
       <c r="Z17" s="6" t="inlineStr">
         <is>
@@ -28204,7 +28228,7 @@
       </c>
       <c r="AL17" s="10" t="inlineStr"/>
       <c r="AM17" s="16" t="n">
-        <v>0</v>
+        <v>0.1644534113375159</v>
       </c>
       <c r="AN17" s="54" t="n">
         <v>1</v>
@@ -28225,24 +28249,26 @@
         <v>75</v>
       </c>
       <c r="AT17" s="58" t="n">
-        <v>0.0039</v>
+        <v>0.006200000000000001</v>
       </c>
       <c r="AU17" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV17" s="17" t="n">
-        <v>4732165.0821</v>
-      </c>
-      <c r="AW17" s="58" t="n"/>
+        <v>6010568.723499999</v>
+      </c>
+      <c r="AW17" s="58" t="n">
+        <v>0.06086427267193487</v>
+      </c>
       <c r="AX17" s="14" t="inlineStr"/>
       <c r="AY17" s="20" t="n">
-        <v>0.1639</v>
+        <v>0.16446</v>
       </c>
       <c r="AZ17" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA17" s="61" t="n">
-        <v>1.639</v>
+        <v>1.643</v>
       </c>
       <c r="BB17" s="60" t="n">
         <v>0.0001</v>
@@ -28263,10 +28289,10 @@
         <v>8</v>
       </c>
       <c r="BH17" s="21" t="n">
-        <v>1165898.641</v>
+        <v>1148657.505</v>
       </c>
       <c r="BI17" s="64" t="n">
-        <v>0.06101281269067526</v>
+        <v>0.06086427267193487</v>
       </c>
       <c r="BJ17" s="18" t="inlineStr">
         <is>
@@ -28274,13 +28300,13 @@
         </is>
       </c>
       <c r="BK17" s="24" t="n">
-        <v>0.16405</v>
+        <v>0.16445</v>
       </c>
       <c r="BL17" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM17" s="67" t="n">
-        <v>0.163955</v>
+        <v>0.16437</v>
       </c>
       <c r="BN17" s="66" t="n"/>
       <c r="BO17" s="68" t="n"/>
@@ -28291,16 +28317,16 @@
         <v>10</v>
       </c>
       <c r="BR17" s="70" t="n">
-        <v>0.00026645</v>
+        <v>0.00125</v>
       </c>
       <c r="BS17" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT17" s="25" t="n">
-        <v>455250.0047399999</v>
+        <v>433619.48817</v>
       </c>
       <c r="BU17" s="70" t="n">
-        <v>0.01219846909212421</v>
+        <v>0.01216767049947816</v>
       </c>
       <c r="BV17" s="22" t="inlineStr">
         <is>
@@ -28356,13 +28382,13 @@
         </is>
       </c>
       <c r="O18" s="8" t="n">
-        <v>0.17201</v>
+        <v>0.17264</v>
       </c>
       <c r="P18" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q18" s="43" t="n">
-        <v>1.7201</v>
+        <v>1.7264</v>
       </c>
       <c r="R18" s="42" t="n">
         <v>1e-05</v>
@@ -28377,16 +28403,16 @@
         <v>50</v>
       </c>
       <c r="V18" s="46" t="n">
-        <v>-0.009183192180489999</v>
+        <v>-0.00864463903395</v>
       </c>
       <c r="W18" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X18" s="9" t="n">
-        <v>567859.1377000001</v>
+        <v>615794.5069</v>
       </c>
       <c r="Y18" s="46" t="n">
-        <v>0.005813615487461337</v>
+        <v>0.00579240037070334</v>
       </c>
       <c r="Z18" s="6" t="inlineStr">
         <is>
@@ -28406,7 +28432,7 @@
       <c r="AK18" s="52" t="n"/>
       <c r="AL18" s="10" t="inlineStr"/>
       <c r="AM18" s="16" t="n">
-        <v>0</v>
+        <v>0.1726554899729357</v>
       </c>
       <c r="AN18" s="54" t="n">
         <v>1</v>
@@ -28427,24 +28453,26 @@
         <v>75</v>
       </c>
       <c r="AT18" s="58" t="n">
-        <v>-0.007399999999999999</v>
+        <v>-0.0081</v>
       </c>
       <c r="AU18" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV18" s="17" t="n">
-        <v>133483.12347</v>
-      </c>
-      <c r="AW18" s="58" t="n"/>
+        <v>767289.6240000005</v>
+      </c>
+      <c r="AW18" s="58" t="n">
+        <v>0.005797773654922311</v>
+      </c>
       <c r="AX18" s="14" t="inlineStr"/>
       <c r="AY18" s="20" t="n">
-        <v>0.172248</v>
+        <v>0.172795</v>
       </c>
       <c r="AZ18" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA18" s="61" t="n">
-        <v>1.7216</v>
+        <v>1.7266</v>
       </c>
       <c r="BB18" s="60" t="n">
         <v>1e-05</v>
@@ -28459,16 +28487,16 @@
         <v>75</v>
       </c>
       <c r="BF18" s="64" t="n">
-        <v>-0.0026</v>
+        <v>-0.0059</v>
       </c>
       <c r="BG18" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH18" s="21" t="n">
-        <v>230660.4422</v>
+        <v>245805.9304</v>
       </c>
       <c r="BI18" s="64" t="n">
-        <v>0.02323420074350154</v>
+        <v>0.03475037646241428</v>
       </c>
       <c r="BJ18" s="18" t="inlineStr">
         <is>
@@ -28476,13 +28504,13 @@
         </is>
       </c>
       <c r="BK18" s="24" t="n">
-        <v>0.17245</v>
+        <v>0.17265</v>
       </c>
       <c r="BL18" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM18" s="67" t="n">
-        <v>0.17234</v>
+        <v>0.17252</v>
       </c>
       <c r="BN18" s="66" t="n"/>
       <c r="BO18" s="68" t="n"/>
@@ -28493,16 +28521,16 @@
         <v>5</v>
       </c>
       <c r="BR18" s="70" t="n">
-        <v>-0.00059187</v>
+        <v>-0.00178583</v>
       </c>
       <c r="BS18" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT18" s="25" t="n">
-        <v>127250.4188</v>
+        <v>130065.50691</v>
       </c>
       <c r="BU18" s="70" t="n">
-        <v>0.0174074503887677</v>
+        <v>0.005796429399495711</v>
       </c>
       <c r="BV18" s="22" t="inlineStr">
         <is>
@@ -28558,13 +28586,13 @@
         </is>
       </c>
       <c r="O19" s="8" t="n">
-        <v>0.12136</v>
+        <v>0.12207</v>
       </c>
       <c r="P19" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q19" s="43" t="n">
-        <v>1.2136</v>
+        <v>1.2207</v>
       </c>
       <c r="R19" s="42" t="n">
         <v>1e-05</v>
@@ -28585,10 +28613,10 @@
         <v>4</v>
       </c>
       <c r="X19" s="9" t="n">
-        <v>80443.36729999997</v>
+        <v>80078.08730000003</v>
       </c>
       <c r="Y19" s="46" t="n">
-        <v>0.008239947264345749</v>
+        <v>0.01638404194314102</v>
       </c>
       <c r="Z19" s="6" t="inlineStr">
         <is>
@@ -28630,7 +28658,7 @@
       </c>
       <c r="AL19" s="10" t="inlineStr"/>
       <c r="AM19" s="16" t="n">
-        <v>0</v>
+        <v>0.122398</v>
       </c>
       <c r="AN19" s="54" t="n">
         <v>1</v>
@@ -28651,24 +28679,26 @@
         <v>20</v>
       </c>
       <c r="AT19" s="58" t="n">
-        <v>-0.0007</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="AU19" s="59" t="n">
         <v>4</v>
       </c>
       <c r="AV19" s="17" t="n">
-        <v>149758.31299</v>
-      </c>
-      <c r="AW19" s="58" t="n"/>
+        <v>191119.41668</v>
+      </c>
+      <c r="AW19" s="58" t="n">
+        <v>0.05734884483041178</v>
+      </c>
       <c r="AX19" s="14" t="inlineStr"/>
       <c r="AY19" s="20" t="n">
-        <v>0.121455</v>
+        <v>0.122212</v>
       </c>
       <c r="AZ19" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA19" s="61" t="n">
-        <v>1.2133</v>
+        <v>1.2198</v>
       </c>
       <c r="BB19" s="60" t="n">
         <v>1e-05</v>
@@ -28689,10 +28719,10 @@
         <v>4</v>
       </c>
       <c r="BH19" s="21" t="n">
-        <v>37802.6764</v>
+        <v>29364.4222</v>
       </c>
       <c r="BI19" s="64" t="n">
-        <v>0.04120992334953803</v>
+        <v>0.1557632398753859</v>
       </c>
       <c r="BJ19" s="18" t="inlineStr">
         <is>
@@ -28700,13 +28730,13 @@
         </is>
       </c>
       <c r="BK19" s="24" t="n">
-        <v>0.121583</v>
+        <v>0.122405</v>
       </c>
       <c r="BL19" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM19" s="67" t="n">
-        <v>0.12156</v>
+        <v>0.122322</v>
       </c>
       <c r="BN19" s="66" t="n"/>
       <c r="BO19" s="68" t="n"/>
@@ -28717,16 +28747,16 @@
         <v>3</v>
       </c>
       <c r="BR19" s="70" t="n">
-        <v>0.00125</v>
+        <v>0.00108342</v>
       </c>
       <c r="BS19" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT19" s="25" t="n">
-        <v>61257.0017</v>
+        <v>57709.30030000001</v>
       </c>
       <c r="BU19" s="70" t="n">
-        <v>0.008226390259950743</v>
+        <v>0.04905086574778413</v>
       </c>
       <c r="BV19" s="22" t="inlineStr">
         <is>
@@ -28866,13 +28896,13 @@
         </is>
       </c>
       <c r="O21" s="8" t="n">
-        <v>209.6</v>
+        <v>210.6</v>
       </c>
       <c r="P21" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q21" s="43" t="n">
-        <v>2.096000000000001</v>
+        <v>2.106</v>
       </c>
       <c r="R21" s="42" t="n">
         <v>0.1</v>
@@ -28893,10 +28923,10 @@
         <v>8</v>
       </c>
       <c r="X21" s="9" t="n">
-        <v>983909.9890000002</v>
+        <v>1031869.127</v>
       </c>
       <c r="Y21" s="46" t="n">
-        <v>0.04770992366411943</v>
+        <v>0.04748338081671145</v>
       </c>
       <c r="Z21" s="6" t="inlineStr">
         <is>
@@ -28938,7 +28968,7 @@
       </c>
       <c r="AL21" s="10" t="inlineStr"/>
       <c r="AM21" s="16" t="n">
-        <v>0</v>
+        <v>210.8969610664052</v>
       </c>
       <c r="AN21" s="54" t="n">
         <v>0.01</v>
@@ -28965,18 +28995,20 @@
         <v>8</v>
       </c>
       <c r="AV21" s="17" t="n">
-        <v>123694.3951</v>
-      </c>
-      <c r="AW21" s="58" t="n"/>
+        <v>470123.0428</v>
+      </c>
+      <c r="AW21" s="58" t="n">
+        <v>0.004744958481622457</v>
+      </c>
       <c r="AX21" s="14" t="inlineStr"/>
       <c r="AY21" s="20" t="n">
-        <v>209.8</v>
+        <v>210.85</v>
       </c>
       <c r="AZ21" s="60" t="n">
         <v>0.01</v>
       </c>
       <c r="BA21" s="61" t="n">
-        <v>2.0981</v>
+        <v>2.1082</v>
       </c>
       <c r="BB21" s="60" t="n">
         <v>0.01</v>
@@ -28991,16 +29023,16 @@
         <v>75</v>
       </c>
       <c r="BF21" s="64" t="n">
-        <v>0.01</v>
+        <v>0.0025</v>
       </c>
       <c r="BG21" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH21" s="21" t="n">
-        <v>536094.1097000001</v>
+        <v>603505.4383999999</v>
       </c>
       <c r="BI21" s="64" t="n">
-        <v>0.03812973642818936</v>
+        <v>0.02846029788445227</v>
       </c>
       <c r="BJ21" s="18" t="inlineStr">
         <is>
@@ -29008,13 +29040,13 @@
         </is>
       </c>
       <c r="BK21" s="24" t="n">
-        <v>210.04</v>
+        <v>210.89</v>
       </c>
       <c r="BL21" s="66" t="n">
         <v>0.001</v>
       </c>
       <c r="BM21" s="67" t="n">
-        <v>0.20991</v>
+        <v>0.21076</v>
       </c>
       <c r="BN21" s="66" t="n"/>
       <c r="BO21" s="68" t="n"/>
@@ -29025,16 +29057,16 @@
         <v>10</v>
       </c>
       <c r="BR21" s="70" t="n">
-        <v>0.00125</v>
+        <v>0.00034817</v>
       </c>
       <c r="BS21" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT21" s="25" t="n">
-        <v>180544.1288</v>
+        <v>128151.3388</v>
       </c>
       <c r="BU21" s="70" t="n">
-        <v>0.01905578581297721</v>
+        <v>0.004744733345995126</v>
       </c>
       <c r="BV21" s="22" t="inlineStr">
         <is>
@@ -29123,13 +29155,13 @@
         <v>50</v>
       </c>
       <c r="BF22" s="64" t="n">
-        <v>-0.0005</v>
+        <v>-0.0024</v>
       </c>
       <c r="BG22" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH22" s="21" t="n">
-        <v>70636.7602</v>
+        <v>69998.64349999999</v>
       </c>
       <c r="BI22" s="64" t="n">
         <v>0.1301561874249067</v>
@@ -29200,13 +29232,13 @@
         </is>
       </c>
       <c r="O23" s="8" t="n">
-        <v>1.419</v>
+        <v>1.421</v>
       </c>
       <c r="P23" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q23" s="43" t="n">
-        <v>1.419</v>
+        <v>1.421</v>
       </c>
       <c r="R23" s="42" t="n">
         <v>0.001</v>
@@ -29227,10 +29259,10 @@
         <v>4</v>
       </c>
       <c r="X23" s="9" t="n">
-        <v>509579.2820000001</v>
+        <v>478318.204</v>
       </c>
       <c r="Y23" s="46" t="n">
-        <v>0.07047216349541155</v>
+        <v>0.07037297677690992</v>
       </c>
       <c r="Z23" s="6" t="inlineStr">
         <is>
@@ -29272,7 +29304,7 @@
       </c>
       <c r="AL23" s="10" t="inlineStr"/>
       <c r="AM23" s="16" t="n">
-        <v>0</v>
+        <v>1.422602436393691</v>
       </c>
       <c r="AN23" s="54" t="n">
         <v>0.1</v>
@@ -29299,18 +29331,20 @@
         <v>4</v>
       </c>
       <c r="AV23" s="17" t="n">
-        <v>117932.12599</v>
-      </c>
-      <c r="AW23" s="58" t="n"/>
+        <v>215927.10637</v>
+      </c>
+      <c r="AW23" s="58" t="n">
+        <v>0.02110595187842739</v>
+      </c>
       <c r="AX23" s="14" t="inlineStr"/>
       <c r="AY23" s="20" t="n">
-        <v>1.42278</v>
+        <v>1.42317</v>
       </c>
       <c r="AZ23" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA23" s="61" t="n">
-        <v>1.4214</v>
+        <v>1.4225</v>
       </c>
       <c r="BB23" s="60" t="n">
         <v>0.0001</v>
@@ -29325,16 +29359,16 @@
         <v>75</v>
       </c>
       <c r="BF23" s="64" t="n">
-        <v>-0.02</v>
+        <v>-0.0038</v>
       </c>
       <c r="BG23" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH23" s="21" t="n">
-        <v>215963.5435999999</v>
+        <v>213429.5235000001</v>
       </c>
       <c r="BI23" s="64" t="n">
-        <v>0.06331785563528218</v>
+        <v>0.06326889279438473</v>
       </c>
       <c r="BJ23" s="18" t="inlineStr">
         <is>
@@ -29342,13 +29376,13 @@
         </is>
       </c>
       <c r="BK23" s="24" t="n">
-        <v>1.423725</v>
+        <v>1.423</v>
       </c>
       <c r="BL23" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM23" s="67" t="n">
-        <v>1.4225</v>
+        <v>1.4219</v>
       </c>
       <c r="BN23" s="66" t="n"/>
       <c r="BO23" s="68" t="n"/>
@@ -29365,10 +29399,10 @@
         <v>1</v>
       </c>
       <c r="BT23" s="25" t="n">
-        <v>105270.6151</v>
+        <v>100990.8469</v>
       </c>
       <c r="BU23" s="70" t="n">
-        <v>0.0281195079086085</v>
+        <v>0.04922990365004029</v>
       </c>
       <c r="BV23" s="22" t="inlineStr">
         <is>
@@ -29508,13 +29542,13 @@
         </is>
       </c>
       <c r="O25" s="8" t="n">
-        <v>45.28</v>
+        <v>45.27</v>
       </c>
       <c r="P25" s="42" t="n">
         <v>0.1</v>
       </c>
       <c r="Q25" s="43" t="n">
-        <v>4.528</v>
+        <v>4.527</v>
       </c>
       <c r="R25" s="42" t="n">
         <v>0.01</v>
@@ -29529,16 +29563,16 @@
         <v>50</v>
       </c>
       <c r="V25" s="46" t="n">
-        <v>-0.0034551061859</v>
+        <v>0.00285093378167</v>
       </c>
       <c r="W25" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X25" s="9" t="n">
-        <v>2701127.919999999</v>
+        <v>2703049.779</v>
       </c>
       <c r="Y25" s="46" t="n">
-        <v>0.02208480565370585</v>
+        <v>0.02208968411751272</v>
       </c>
       <c r="Z25" s="6" t="inlineStr">
         <is>
@@ -29580,7 +29614,7 @@
       </c>
       <c r="AL25" s="10" t="inlineStr"/>
       <c r="AM25" s="16" t="n">
-        <v>0</v>
+        <v>45.30464456064654</v>
       </c>
       <c r="AN25" s="54" t="n">
         <v>0.1</v>
@@ -29601,24 +29635,26 @@
         <v>75</v>
       </c>
       <c r="AT25" s="58" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.0046</v>
       </c>
       <c r="AU25" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV25" s="17" t="n">
-        <v>2394593.191999999</v>
-      </c>
-      <c r="AW25" s="58" t="n"/>
+        <v>4129793.482000003</v>
+      </c>
+      <c r="AW25" s="58" t="n">
+        <v>0.02208480565370585</v>
+      </c>
       <c r="AX25" s="14" t="inlineStr"/>
       <c r="AY25" s="20" t="n">
-        <v>45.34</v>
+        <v>45.31</v>
       </c>
       <c r="AZ25" s="60" t="n">
         <v>0.1</v>
       </c>
       <c r="BA25" s="61" t="n">
-        <v>4.531000000000001</v>
+        <v>4.528</v>
       </c>
       <c r="BB25" s="60" t="n">
         <v>0.01</v>
@@ -29639,10 +29675,10 @@
         <v>8</v>
       </c>
       <c r="BH25" s="21" t="n">
-        <v>659002.5119999999</v>
+        <v>665642.1669999999</v>
       </c>
       <c r="BI25" s="64" t="n">
-        <v>0.02207018318253171</v>
+        <v>0.02208480565370585</v>
       </c>
       <c r="BJ25" s="18" t="inlineStr">
         <is>
@@ -29650,13 +29686,13 @@
         </is>
       </c>
       <c r="BK25" s="24" t="n">
-        <v>45.345</v>
+        <v>45.305</v>
       </c>
       <c r="BL25" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM25" s="67" t="n">
-        <v>0.45318</v>
+        <v>0.452781</v>
       </c>
       <c r="BN25" s="66" t="n"/>
       <c r="BO25" s="68" t="n"/>
@@ -29667,16 +29703,16 @@
         <v>10</v>
       </c>
       <c r="BR25" s="70" t="n">
-        <v>0.0007093399999999999</v>
+        <v>0.00059238</v>
       </c>
       <c r="BS25" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT25" s="25" t="n">
-        <v>108206.18986</v>
+        <v>119702.26237</v>
       </c>
       <c r="BU25" s="70" t="n">
-        <v>0.006619886137958678</v>
+        <v>0.00220857323961203</v>
       </c>
       <c r="BV25" s="22" t="inlineStr">
         <is>
@@ -29816,13 +29852,13 @@
         </is>
       </c>
       <c r="O27" s="8" t="n">
-        <v>0.06789000000000001</v>
+        <v>0.06777</v>
       </c>
       <c r="P27" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q27" s="43" t="n">
-        <v>0.6789000000000001</v>
+        <v>0.6777</v>
       </c>
       <c r="R27" s="42" t="n">
         <v>1e-05</v>
@@ -29843,10 +29879,10 @@
         <v>8</v>
       </c>
       <c r="X27" s="9" t="n">
-        <v>974431.3771999999</v>
+        <v>1014785.6461</v>
       </c>
       <c r="Y27" s="46" t="n">
-        <v>0.01472970982473118</v>
+        <v>0.01475579164823668</v>
       </c>
       <c r="Z27" s="6" t="inlineStr">
         <is>
@@ -29888,7 +29924,7 @@
       </c>
       <c r="AL27" s="10" t="inlineStr"/>
       <c r="AM27" s="16" t="n">
-        <v>0</v>
+        <v>0.06783259282300411</v>
       </c>
       <c r="AN27" s="54" t="n">
         <v>1</v>
@@ -29909,24 +29945,26 @@
         <v>75</v>
       </c>
       <c r="AT27" s="58" t="n">
-        <v>0.007600000000000001</v>
+        <v>0.0069</v>
       </c>
       <c r="AU27" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV27" s="17" t="n">
-        <v>722814.0282300003</v>
-      </c>
-      <c r="AW27" s="58" t="n"/>
+        <v>1710895.52009</v>
+      </c>
+      <c r="AW27" s="58" t="n">
+        <v>0.01475361463558</v>
+      </c>
       <c r="AX27" s="14" t="inlineStr"/>
       <c r="AY27" s="20" t="n">
-        <v>0.06794699999999999</v>
+        <v>0.067857</v>
       </c>
       <c r="AZ27" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA27" s="61" t="n">
-        <v>0.6795</v>
+        <v>0.6784999999999999</v>
       </c>
       <c r="BB27" s="60" t="n">
         <v>1e-05</v>
@@ -29947,10 +29985,10 @@
         <v>8</v>
       </c>
       <c r="BH27" s="21" t="n">
-        <v>222445.4982999999</v>
+        <v>204233.8075</v>
       </c>
       <c r="BI27" s="64" t="n">
-        <v>0.02943340691685964</v>
+        <v>0.02947678703022273</v>
       </c>
       <c r="BJ27" s="18" t="inlineStr">
         <is>
@@ -29958,13 +29996,13 @@
         </is>
       </c>
       <c r="BK27" s="24" t="n">
-        <v>0.068</v>
+        <v>0.067815</v>
       </c>
       <c r="BL27" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM27" s="67" t="n">
-        <v>0.06794500000000001</v>
+        <v>0.067745</v>
       </c>
       <c r="BN27" s="66" t="n"/>
       <c r="BO27" s="68" t="n"/>
@@ -29975,16 +30013,16 @@
         <v>5</v>
       </c>
       <c r="BR27" s="70" t="n">
-        <v>0.00052474</v>
+        <v>0.0002055</v>
       </c>
       <c r="BS27" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT27" s="25" t="n">
-        <v>92249.64912799999</v>
+        <v>76252.86191500002</v>
       </c>
       <c r="BU27" s="70" t="n">
-        <v>0.01766134373389966</v>
+        <v>0.008856742194984312</v>
       </c>
       <c r="BV27" s="22" t="inlineStr">
         <is>
@@ -30040,13 +30078,13 @@
         </is>
       </c>
       <c r="O28" s="8" t="n">
-        <v>0.6867</v>
+        <v>0.6906</v>
       </c>
       <c r="P28" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q28" s="43" t="n">
-        <v>0.6867</v>
+        <v>0.6906</v>
       </c>
       <c r="R28" s="42" t="n">
         <v>0.0001</v>
@@ -30067,10 +30105,10 @@
         <v>8</v>
       </c>
       <c r="X28" s="9" t="n">
-        <v>2179461.319600001</v>
+        <v>1889828.622</v>
       </c>
       <c r="Y28" s="46" t="n">
-        <v>0.0145623998834992</v>
+        <v>0.0144801621778148</v>
       </c>
       <c r="Z28" s="6" t="inlineStr">
         <is>
@@ -30090,7 +30128,7 @@
       <c r="AK28" s="52" t="n"/>
       <c r="AL28" s="10" t="inlineStr"/>
       <c r="AM28" s="16" t="n">
-        <v>0</v>
+        <v>0.6911038026472314</v>
       </c>
       <c r="AN28" s="54" t="n">
         <v>0.1</v>
@@ -30117,18 +30155,20 @@
         <v>8</v>
       </c>
       <c r="AV28" s="17" t="n">
-        <v>1902642.54052</v>
-      </c>
-      <c r="AW28" s="58" t="n"/>
+        <v>3356888.59763</v>
+      </c>
+      <c r="AW28" s="58" t="n">
+        <v>0.01447806573041682</v>
+      </c>
       <c r="AX28" s="14" t="inlineStr"/>
       <c r="AY28" s="20" t="n">
-        <v>0.6876</v>
+        <v>0.69085</v>
       </c>
       <c r="AZ28" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA28" s="61" t="n">
-        <v>0.6876</v>
+        <v>0.6904</v>
       </c>
       <c r="BB28" s="60" t="n">
         <v>0.0001</v>
@@ -30143,16 +30183,16 @@
         <v>50</v>
       </c>
       <c r="BF28" s="64" t="n">
-        <v>0.009399999999999999</v>
+        <v>0.0083</v>
       </c>
       <c r="BG28" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH28" s="21" t="n">
-        <v>772328.0706000002</v>
+        <v>655915.13</v>
       </c>
       <c r="BI28" s="64" t="n">
-        <v>0.01454333915066739</v>
+        <v>0.01448435689455228</v>
       </c>
       <c r="BJ28" s="18" t="inlineStr">
         <is>
@@ -30160,13 +30200,13 @@
         </is>
       </c>
       <c r="BK28" s="24" t="n">
-        <v>0.6883</v>
+        <v>0.6910500000000001</v>
       </c>
       <c r="BL28" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM28" s="67" t="n">
-        <v>0.06879</v>
+        <v>0.069079</v>
       </c>
       <c r="BN28" s="66" t="n"/>
       <c r="BO28" s="68" t="n"/>
@@ -30183,10 +30223,10 @@
         <v>1</v>
       </c>
       <c r="BT28" s="25" t="n">
-        <v>152956.707001</v>
+        <v>194615.909743</v>
       </c>
       <c r="BU28" s="70" t="n">
-        <v>0.0014536996656586</v>
+        <v>0.004342853834012434</v>
       </c>
       <c r="BV28" s="22" t="inlineStr">
         <is>
@@ -30242,13 +30282,13 @@
         </is>
       </c>
       <c r="O29" s="8" t="n">
-        <v>6.419</v>
+        <v>6.457</v>
       </c>
       <c r="P29" s="42" t="n">
         <v>0.1</v>
       </c>
       <c r="Q29" s="43" t="n">
-        <v>0.6419</v>
+        <v>0.6457000000000001</v>
       </c>
       <c r="R29" s="42" t="n">
         <v>0.001</v>
@@ -30263,16 +30303,16 @@
         <v>50</v>
       </c>
       <c r="V29" s="46" t="n">
-        <v>0.00415040943632</v>
+        <v>-0.00177598999323</v>
       </c>
       <c r="W29" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X29" s="9" t="n">
-        <v>1401829.8908</v>
+        <v>1462744.7648</v>
       </c>
       <c r="Y29" s="46" t="n">
-        <v>0.01557875058420835</v>
+        <v>0.01548706829796261</v>
       </c>
       <c r="Z29" s="6" t="inlineStr">
         <is>
@@ -30314,7 +30354,7 @@
       </c>
       <c r="AL29" s="10" t="inlineStr"/>
       <c r="AM29" s="16" t="n">
-        <v>0</v>
+        <v>6.465498740614327</v>
       </c>
       <c r="AN29" s="54" t="n">
         <v>0.1</v>
@@ -30335,24 +30375,26 @@
         <v>75</v>
       </c>
       <c r="AT29" s="58" t="n">
-        <v>0.0039</v>
+        <v>0.01</v>
       </c>
       <c r="AU29" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV29" s="17" t="n">
-        <v>1054010.2601</v>
-      </c>
-      <c r="AW29" s="58" t="n"/>
+        <v>2041793.021600001</v>
+      </c>
+      <c r="AW29" s="58" t="n">
+        <v>0.01547508511297329</v>
+      </c>
       <c r="AX29" s="14" t="inlineStr"/>
       <c r="AY29" s="20" t="n">
-        <v>6.4277</v>
+        <v>6.4638</v>
       </c>
       <c r="AZ29" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA29" s="61" t="n">
-        <v>6.426</v>
+        <v>6.46</v>
       </c>
       <c r="BB29" s="60" t="n">
         <v>0.001</v>
@@ -30367,16 +30409,16 @@
         <v>75</v>
       </c>
       <c r="BF29" s="64" t="n">
-        <v>0.009399999999999999</v>
+        <v>0.0014</v>
       </c>
       <c r="BG29" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH29" s="21" t="n">
-        <v>1007990.132</v>
+        <v>889044.9249999999</v>
       </c>
       <c r="BI29" s="64" t="n">
-        <v>0.03112356053532181</v>
+        <v>0.01547987616099588</v>
       </c>
       <c r="BJ29" s="18" t="inlineStr">
         <is>
@@ -30384,13 +30426,13 @@
         </is>
       </c>
       <c r="BK29" s="24" t="n">
-        <v>6.4325</v>
+        <v>6.4656</v>
       </c>
       <c r="BL29" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM29" s="67" t="n">
-        <v>0.064291</v>
+        <v>0.06461</v>
       </c>
       <c r="BN29" s="66" t="n"/>
       <c r="BO29" s="68" t="n"/>
@@ -30401,16 +30443,16 @@
         <v>10</v>
       </c>
       <c r="BR29" s="70" t="n">
-        <v>0.00114378</v>
+        <v>-0.00049734</v>
       </c>
       <c r="BS29" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT29" s="25" t="n">
-        <v>80151.709754</v>
+        <v>65077.795532</v>
       </c>
       <c r="BU29" s="70" t="n">
-        <v>0.007777138324177924</v>
+        <v>0.001547748026617659</v>
       </c>
       <c r="BV29" s="22" t="inlineStr">
         <is>
@@ -30442,13 +30484,13 @@
       <c r="M30" s="40" t="n"/>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="8" t="n">
-        <v>4.588e-06</v>
+        <v>4.619e-06</v>
       </c>
       <c r="P30" s="42" t="n">
         <v>100000</v>
       </c>
       <c r="Q30" s="43" t="n">
-        <v>0.4588</v>
+        <v>0.4619</v>
       </c>
       <c r="R30" s="42" t="n">
         <v>1e-09</v>
@@ -30463,16 +30505,16 @@
         <v>50</v>
       </c>
       <c r="V30" s="46" t="n">
-        <v>0.00853882245563</v>
+        <v>0.009645496793820001</v>
       </c>
       <c r="W30" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X30" s="9" t="n">
-        <v>1622276.7063</v>
+        <v>1752230.3716</v>
       </c>
       <c r="Y30" s="46" t="n">
-        <v>0.02179598953793589</v>
+        <v>0.02164970772893812</v>
       </c>
       <c r="Z30" s="6" t="inlineStr">
         <is>
@@ -30492,7 +30534,7 @@
       <c r="AK30" s="52" t="n"/>
       <c r="AL30" s="10" t="inlineStr"/>
       <c r="AM30" s="16" t="n">
-        <v>0</v>
+        <v>4.6200415498e-06</v>
       </c>
       <c r="AN30" s="54" t="n">
         <v>10000</v>
@@ -30519,18 +30561,20 @@
         <v>8</v>
       </c>
       <c r="AV30" s="17" t="n">
-        <v>2090162.11718</v>
-      </c>
-      <c r="AW30" s="58" t="n"/>
+        <v>3211414.26259</v>
+      </c>
+      <c r="AW30" s="58" t="n">
+        <v>0.0216543958423668</v>
+      </c>
       <c r="AX30" s="14" t="inlineStr"/>
       <c r="AY30" s="20" t="n">
-        <v>4.597e-06</v>
+        <v>4.621e-06</v>
       </c>
       <c r="AZ30" s="60" t="n">
         <v>10000</v>
       </c>
       <c r="BA30" s="61" t="n">
-        <v>0.04597</v>
+        <v>0.04619</v>
       </c>
       <c r="BB30" s="60" t="n">
         <v>1e-09</v>
@@ -30545,16 +30589,16 @@
         <v>75</v>
       </c>
       <c r="BF30" s="64" t="n">
-        <v>0.01</v>
+        <v>0.0091</v>
       </c>
       <c r="BG30" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH30" s="21" t="n">
-        <v>885753.9166499999</v>
+        <v>749699.27174</v>
       </c>
       <c r="BI30" s="64" t="n">
-        <v>0.04350663476180444</v>
+        <v>0.04329941545787623</v>
       </c>
       <c r="BJ30" s="18" t="inlineStr">
         <is>
@@ -30682,13 +30726,13 @@
       <c r="M32" s="40" t="n"/>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="8" t="n">
-        <v>0.05476</v>
+        <v>0.0551</v>
       </c>
       <c r="P32" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q32" s="43" t="n">
-        <v>0.5476000000000001</v>
+        <v>0.551</v>
       </c>
       <c r="R32" s="42" t="n">
         <v>1e-05</v>
@@ -30709,10 +30753,10 @@
         <v>8</v>
       </c>
       <c r="X32" s="9" t="n">
-        <v>111463.4424</v>
+        <v>107652.8943</v>
       </c>
       <c r="Y32" s="46" t="n">
-        <v>0.01826150474799683</v>
+        <v>0.01814882032667173</v>
       </c>
       <c r="Z32" s="6" t="inlineStr">
         <is>
@@ -30754,7 +30798,7 @@
       </c>
       <c r="AL32" s="10" t="inlineStr"/>
       <c r="AM32" s="16" t="n">
-        <v>0</v>
+        <v>0.055193684877192</v>
       </c>
       <c r="AN32" s="54" t="n">
         <v>1</v>
@@ -30781,18 +30825,20 @@
         <v>8</v>
       </c>
       <c r="AV32" s="17" t="n">
-        <v>99408.89286000002</v>
-      </c>
-      <c r="AW32" s="58" t="n"/>
+        <v>127325.01877</v>
+      </c>
+      <c r="AW32" s="58" t="n">
+        <v>0.07249003262051174</v>
+      </c>
       <c r="AX32" s="14" t="inlineStr"/>
       <c r="AY32" s="20" t="n">
-        <v>0.054817</v>
+        <v>0.055191</v>
       </c>
       <c r="AZ32" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA32" s="61" t="n">
-        <v>0.05471</v>
+        <v>0.05507</v>
       </c>
       <c r="BB32" s="60" t="n">
         <v>1e-05</v>
@@ -30807,16 +30853,16 @@
         <v>25</v>
       </c>
       <c r="BF32" s="64" t="n">
-        <v>-0.0026</v>
+        <v>0.01</v>
       </c>
       <c r="BG32" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH32" s="21" t="n">
-        <v>12950.47464</v>
+        <v>12187.31298</v>
       </c>
       <c r="BI32" s="64" t="n">
-        <v>0.07311277645768299</v>
+        <v>0.07263482840021494</v>
       </c>
       <c r="BJ32" s="18" t="inlineStr">
         <is>
@@ -30884,13 +30930,13 @@
         </is>
       </c>
       <c r="O33" s="8" t="n">
-        <v>4.051</v>
+        <v>4.012</v>
       </c>
       <c r="P33" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q33" s="43" t="n">
-        <v>4.051</v>
+        <v>4.012</v>
       </c>
       <c r="R33" s="42" t="n">
         <v>0.001</v>
@@ -30905,16 +30951,16 @@
         <v>50</v>
       </c>
       <c r="V33" s="46" t="n">
-        <v>0.00563952083758</v>
+        <v>0.00055630806879</v>
       </c>
       <c r="W33" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X33" s="9" t="n">
-        <v>1138133.483</v>
+        <v>1166082.457</v>
       </c>
       <c r="Y33" s="46" t="n">
-        <v>0.02468526289803618</v>
+        <v>0.02492522432700513</v>
       </c>
       <c r="Z33" s="6" t="inlineStr">
         <is>
@@ -30934,7 +30980,7 @@
       <c r="AK33" s="52" t="n"/>
       <c r="AL33" s="10" t="inlineStr"/>
       <c r="AM33" s="16" t="n">
-        <v>0</v>
+        <v>4.015995053489071</v>
       </c>
       <c r="AN33" s="54" t="n">
         <v>1</v>
@@ -30961,18 +31007,20 @@
         <v>8</v>
       </c>
       <c r="AV33" s="17" t="n">
-        <v>978269.3299999996</v>
-      </c>
-      <c r="AW33" s="58" t="n"/>
+        <v>1923758.584</v>
+      </c>
+      <c r="AW33" s="58" t="n">
+        <v>0.0498504486540324</v>
+      </c>
       <c r="AX33" s="14" t="inlineStr"/>
       <c r="AY33" s="20" t="n">
-        <v>4.0618</v>
+        <v>4.0154</v>
       </c>
       <c r="AZ33" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA33" s="61" t="n">
-        <v>4.059</v>
+        <v>4.011</v>
       </c>
       <c r="BB33" s="60" t="n">
         <v>0.001</v>
@@ -30987,16 +31035,16 @@
         <v>75</v>
       </c>
       <c r="BF33" s="64" t="n">
-        <v>0.0041</v>
+        <v>0.002</v>
       </c>
       <c r="BG33" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH33" s="21" t="n">
-        <v>463110.713</v>
+        <v>465229.5519999997</v>
       </c>
       <c r="BI33" s="64" t="n">
-        <v>0.02463661000247189</v>
+        <v>0.04986287708802464</v>
       </c>
       <c r="BJ33" s="18" t="inlineStr">
         <is>
@@ -31004,13 +31052,13 @@
         </is>
       </c>
       <c r="BK33" s="24" t="n">
-        <v>4.0555</v>
+        <v>4.0155</v>
       </c>
       <c r="BL33" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM33" s="67" t="n">
-        <v>0.40545</v>
+        <v>0.40149</v>
       </c>
       <c r="BN33" s="66" t="n"/>
       <c r="BO33" s="68" t="n"/>
@@ -31027,10 +31075,10 @@
         <v>1</v>
       </c>
       <c r="BT33" s="25" t="n">
-        <v>100534.00817</v>
+        <v>77071.53523999998</v>
       </c>
       <c r="BU33" s="70" t="n">
-        <v>0.002466395363170969</v>
+        <v>0.002490722060319483</v>
       </c>
       <c r="BV33" s="22" t="inlineStr">
         <is>
@@ -31110,7 +31158,7 @@
       <c r="AK34" s="52" t="n"/>
       <c r="AL34" s="10" t="inlineStr"/>
       <c r="AM34" s="16" t="n">
-        <v>0</v>
+        <v>4059.552718715362</v>
       </c>
       <c r="AN34" s="54" t="n">
         <v>0.01</v>
@@ -31131,24 +31179,26 @@
         <v>75</v>
       </c>
       <c r="AT34" s="58" t="n">
-        <v>0.0041</v>
+        <v>0.002</v>
       </c>
       <c r="AU34" s="59" t="n">
         <v>4</v>
       </c>
       <c r="AV34" s="17" t="n">
-        <v>274610.3951</v>
-      </c>
-      <c r="AW34" s="58" t="n"/>
+        <v>396808.8834999999</v>
+      </c>
+      <c r="AW34" s="58" t="n">
+        <v>0.003696629905738179</v>
+      </c>
       <c r="AX34" s="14" t="inlineStr"/>
       <c r="AY34" s="20" t="n">
-        <v>4055.11</v>
+        <v>4057.91</v>
       </c>
       <c r="AZ34" s="60" t="n">
         <v>0.001</v>
       </c>
       <c r="BA34" s="61" t="n">
-        <v>4.0538</v>
+        <v>4.0563</v>
       </c>
       <c r="BB34" s="60" t="n">
         <v>0.1</v>
@@ -31163,16 +31213,16 @@
         <v>100</v>
       </c>
       <c r="BF34" s="64" t="n">
-        <v>0.0041</v>
+        <v>-0.006</v>
       </c>
       <c r="BG34" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH34" s="21" t="n">
-        <v>690074.2868</v>
+        <v>760109.2137999999</v>
       </c>
       <c r="BI34" s="64" t="n">
-        <v>0.002466821254129682</v>
+        <v>0.002465300889971379</v>
       </c>
       <c r="BJ34" s="18" t="inlineStr">
         <is>
@@ -31200,193 +31250,217 @@
       </c>
       <c r="B35" s="35" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>NEAR</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>193.56743598</v>
+        <v>1.67065676</v>
       </c>
       <c r="D35" s="36" t="n">
-        <v>0.001</v>
+        <v>1</v>
       </c>
       <c r="E35" s="37" t="n">
         <v>5</v>
       </c>
       <c r="F35" s="36" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="G35" s="38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H35" s="36" t="n">
-        <v>0.001</v>
+        <v>1</v>
       </c>
       <c r="I35" s="39" t="n"/>
       <c r="J35" s="40" t="n">
-        <v>0.005</v>
+        <v>-0.009618</v>
       </c>
       <c r="K35" s="41" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>652586.9190799999</v>
+        <v>2069300.265</v>
       </c>
       <c r="M35" s="40" t="n">
-        <v>0.005167799179660471</v>
+        <v>0.05988023952096479</v>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>binance:52%, coinbase:16%, gateio:5%, kucoin:8%, mexc:8%, binance_cross2:4%, bitget:8%</t>
+          <t>binance:54%, okex:16%, gateio:5%, kucoin:8%, mexc:8%, bybit:8%</t>
         </is>
       </c>
       <c r="O35" s="8" t="n">
-        <v>191</v>
+        <v>1.656</v>
       </c>
       <c r="P35" s="42" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="Q35" s="43" t="n">
-        <v>1.91</v>
+        <v>1.656</v>
       </c>
       <c r="R35" s="42" t="n">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
       <c r="S35" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="T35" s="42" t="n">
         <v>1</v>
-      </c>
-      <c r="T35" s="42" t="n">
-        <v>0.01</v>
       </c>
       <c r="U35" s="45" t="n">
         <v>50</v>
       </c>
       <c r="V35" s="46" t="n">
-        <v>0.01</v>
+        <v>-0.01594433248281</v>
       </c>
       <c r="W35" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X35" s="9" t="n">
-        <v>1328791.029</v>
+        <v>1309575.192</v>
       </c>
       <c r="Y35" s="46" t="n">
-        <v>0.0523560209424054</v>
+        <v>0.06038647342994504</v>
       </c>
       <c r="Z35" s="6" t="inlineStr">
         <is>
-          <t>Binance:31%, Coinbase:23%, Bitget:15%, Kucoin:15%, Gate:15%</t>
-        </is>
-      </c>
-      <c r="AA35" s="12" t="n"/>
-      <c r="AB35" s="48" t="n"/>
-      <c r="AC35" s="49" t="n"/>
-      <c r="AD35" s="48" t="n"/>
-      <c r="AE35" s="50" t="n"/>
-      <c r="AF35" s="48" t="n"/>
-      <c r="AG35" s="51" t="n"/>
-      <c r="AH35" s="52" t="n"/>
-      <c r="AI35" s="53" t="n"/>
-      <c r="AJ35" s="13" t="n"/>
-      <c r="AK35" s="52" t="n"/>
+          <t>Binance:27%, Gate:13%, Kucoin:13%, Bybit:20%, OKX:27%</t>
+        </is>
+      </c>
+      <c r="AA35" s="12" t="n">
+        <v>1.6701</v>
+      </c>
+      <c r="AB35" s="48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AC35" s="49" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD35" s="48" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AE35" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF35" s="48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AG35" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH35" s="52" t="n">
+        <v>0.004028</v>
+      </c>
+      <c r="AI35" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ35" s="13" t="n">
+        <v>684761.0835299997</v>
+      </c>
+      <c r="AK35" s="52" t="n">
+        <v>0.005991611743558357</v>
+      </c>
       <c r="AL35" s="10" t="inlineStr"/>
       <c r="AM35" s="16" t="n">
-        <v>0</v>
+        <v>1.659348465896357</v>
       </c>
       <c r="AN35" s="54" t="n">
-        <v>0.001</v>
+        <v>1</v>
       </c>
       <c r="AO35" s="55" t="n">
         <v>5</v>
       </c>
       <c r="AP35" s="54" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="AQ35" s="56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AR35" s="54" t="n">
-        <v>0.001</v>
+        <v>1</v>
       </c>
       <c r="AS35" s="57" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="AT35" s="58" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
       <c r="AU35" s="59" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AV35" s="17" t="n">
-        <v>439756.42933</v>
-      </c>
-      <c r="AW35" s="58" t="n"/>
+        <v>1157577.6939</v>
+      </c>
+      <c r="AW35" s="58" t="n">
+        <v>0.006033182503770074</v>
+      </c>
       <c r="AX35" s="14" t="inlineStr"/>
       <c r="AY35" s="20" t="n">
-        <v>191.28</v>
+        <v>1.6567</v>
       </c>
       <c r="AZ35" s="60" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="BA35" s="61" t="n">
-        <v>1.912</v>
+        <v>1.6552</v>
       </c>
       <c r="BB35" s="60" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="BC35" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="BD35" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE35" s="63" t="n">
+        <v>75</v>
+      </c>
+      <c r="BF35" s="64" t="n">
+        <v>-0.0229</v>
+      </c>
+      <c r="BG35" s="65" t="n">
+        <v>8</v>
+      </c>
+      <c r="BH35" s="21" t="n">
+        <v>221124.6086</v>
+      </c>
+      <c r="BI35" s="64" t="n">
+        <v>0.01812469792169931</v>
+      </c>
+      <c r="BJ35" s="18" t="inlineStr">
+        <is>
+          <t>Binance, Bitget, Bybit, Coinbase, Gate.io, KuCoin, OKX</t>
+        </is>
+      </c>
+      <c r="BK35" s="24" t="n">
+        <v>1.6595</v>
+      </c>
+      <c r="BL35" s="66" t="n">
         <v>0.1</v>
       </c>
-      <c r="BC35" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="BD35" s="60" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="BE35" s="63" t="n">
-        <v>50</v>
-      </c>
-      <c r="BF35" s="64" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="BG35" s="65" t="n">
-        <v>4</v>
-      </c>
-      <c r="BH35" s="21" t="n">
-        <v>188466.95</v>
-      </c>
-      <c r="BI35" s="64" t="n">
-        <v>0.05230125523012255</v>
-      </c>
-      <c r="BJ35" s="18" t="inlineStr">
-        <is>
-          <t>Binance, Bitget, Gate, KuCoin, MEXC, OKX</t>
-        </is>
-      </c>
-      <c r="BK35" s="24" t="n">
-        <v>191.464</v>
-      </c>
-      <c r="BL35" s="66" t="n">
-        <v>0.001</v>
-      </c>
       <c r="BM35" s="67" t="n">
-        <v>0.19142</v>
+        <v>0.16581</v>
       </c>
       <c r="BN35" s="66" t="n"/>
       <c r="BO35" s="68" t="n"/>
       <c r="BP35" s="66" t="n">
-        <v>0.001</v>
+        <v>0.1</v>
       </c>
       <c r="BQ35" s="69" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="BR35" s="70" t="n">
-        <v>0.00125</v>
+        <v>-0.00030172</v>
       </c>
       <c r="BS35" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT35" s="25" t="n">
-        <v>165691.57911</v>
+        <v>250650.39623</v>
       </c>
       <c r="BU35" s="70" t="n">
-        <v>0.0365688015881421</v>
+        <v>0.01206199867317882</v>
       </c>
       <c r="BV35" s="22" t="inlineStr">
         <is>
@@ -31402,215 +31476,195 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>NEAR</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1.67065676</v>
+        <v>193.56743598</v>
       </c>
       <c r="D36" s="36" t="n">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="E36" s="37" t="n">
         <v>5</v>
       </c>
       <c r="F36" s="36" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G36" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" s="36" t="n">
         <v>0.001</v>
-      </c>
-      <c r="G36" s="38" t="n">
-        <v>3</v>
-      </c>
-      <c r="H36" s="36" t="n">
-        <v>1</v>
       </c>
       <c r="I36" s="39" t="n"/>
       <c r="J36" s="40" t="n">
-        <v>-0.009618</v>
+        <v>0.005</v>
       </c>
       <c r="K36" s="41" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>2069300.265</v>
+        <v>652586.9190799999</v>
       </c>
       <c r="M36" s="40" t="n">
-        <v>0.05988023952096479</v>
+        <v>0.005167799179660471</v>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>binance:54%, okex:16%, gateio:5%, kucoin:8%, mexc:8%, bybit:8%</t>
+          <t>binance:52%, coinbase:16%, gateio:5%, kucoin:8%, mexc:8%, binance_cross2:4%, bitget:8%</t>
         </is>
       </c>
       <c r="O36" s="8" t="n">
-        <v>1.623</v>
+        <v>193.3</v>
       </c>
       <c r="P36" s="42" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Q36" s="43" t="n">
+        <v>1.933</v>
+      </c>
+      <c r="R36" s="42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S36" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="Q36" s="43" t="n">
-        <v>1.623</v>
-      </c>
-      <c r="R36" s="42" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="S36" s="44" t="n">
-        <v>3</v>
-      </c>
       <c r="T36" s="42" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="U36" s="45" t="n">
         <v>50</v>
       </c>
       <c r="V36" s="46" t="n">
-        <v>-0.0117064710038</v>
+        <v>0.01</v>
       </c>
       <c r="W36" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X36" s="9" t="n">
-        <v>1215517.604</v>
+        <v>1378102.505</v>
       </c>
       <c r="Y36" s="46" t="n">
-        <v>0.06161429451633468</v>
+        <v>0.0517330574236908</v>
       </c>
       <c r="Z36" s="6" t="inlineStr">
         <is>
-          <t>Binance:27%, Gate:13%, Kucoin:13%, Bybit:20%, OKX:27%</t>
-        </is>
-      </c>
-      <c r="AA36" s="12" t="n">
-        <v>1.6701</v>
-      </c>
-      <c r="AB36" s="48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AC36" s="49" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD36" s="48" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="AE36" s="50" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF36" s="48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AG36" s="51" t="n">
-        <v>50</v>
-      </c>
-      <c r="AH36" s="52" t="n">
-        <v>0.004028</v>
-      </c>
-      <c r="AI36" s="53" t="n">
-        <v>8</v>
-      </c>
-      <c r="AJ36" s="13" t="n">
-        <v>684761.0835299997</v>
-      </c>
-      <c r="AK36" s="52" t="n">
-        <v>0.005991611743558357</v>
-      </c>
+          <t>Binance:31%, Coinbase:23%, Bitget:15%, Kucoin:15%, Gate:15%</t>
+        </is>
+      </c>
+      <c r="AA36" s="12" t="n"/>
+      <c r="AB36" s="48" t="n"/>
+      <c r="AC36" s="49" t="n"/>
+      <c r="AD36" s="48" t="n"/>
+      <c r="AE36" s="50" t="n"/>
+      <c r="AF36" s="48" t="n"/>
+      <c r="AG36" s="51" t="n"/>
+      <c r="AH36" s="52" t="n"/>
+      <c r="AI36" s="53" t="n"/>
+      <c r="AJ36" s="13" t="n"/>
+      <c r="AK36" s="52" t="n"/>
       <c r="AL36" s="10" t="inlineStr"/>
       <c r="AM36" s="16" t="n">
-        <v>0</v>
+        <v>193.410218863788</v>
       </c>
       <c r="AN36" s="54" t="n">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="AO36" s="55" t="n">
         <v>5</v>
       </c>
       <c r="AP36" s="54" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="AQ36" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR36" s="54" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="AS36" s="57" t="n">
+        <v>50</v>
+      </c>
+      <c r="AT36" s="58" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="AU36" s="59" t="n">
         <v>4</v>
       </c>
-      <c r="AR36" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS36" s="57" t="n">
-        <v>75</v>
-      </c>
-      <c r="AT36" s="58" t="n">
-        <v>0.0027</v>
-      </c>
-      <c r="AU36" s="59" t="n">
-        <v>8</v>
-      </c>
       <c r="AV36" s="17" t="n">
-        <v>659444.6461</v>
-      </c>
-      <c r="AW36" s="58" t="n"/>
+        <v>842651.0721000001</v>
+      </c>
+      <c r="AW36" s="58" t="n">
+        <v>0.005173305742379372</v>
+      </c>
       <c r="AX36" s="14" t="inlineStr"/>
       <c r="AY36" s="20" t="n">
-        <v>1.626</v>
+        <v>193.48</v>
       </c>
       <c r="AZ36" s="60" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="BA36" s="61" t="n">
+        <v>1.933</v>
+      </c>
+      <c r="BB36" s="60" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="BC36" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="BA36" s="61" t="n">
-        <v>1.6249</v>
-      </c>
-      <c r="BB36" s="60" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="BC36" s="62" t="n">
+      <c r="BD36" s="60" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="BE36" s="63" t="n">
+        <v>50</v>
+      </c>
+      <c r="BF36" s="64" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="BG36" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="BD36" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE36" s="63" t="n">
-        <v>75</v>
-      </c>
-      <c r="BF36" s="64" t="n">
-        <v>-0.0262</v>
-      </c>
-      <c r="BG36" s="65" t="n">
-        <v>8</v>
-      </c>
       <c r="BH36" s="21" t="n">
-        <v>195695.1588000001</v>
+        <v>184659.143</v>
       </c>
       <c r="BI36" s="64" t="n">
-        <v>0.03077112437688134</v>
+        <v>0.0517330574237055</v>
       </c>
       <c r="BJ36" s="18" t="inlineStr">
         <is>
-          <t>Binance, Bitget, Bybit, Coinbase, Gate.io, KuCoin, OKX</t>
+          <t>Binance, Bitget, Gate, KuCoin, MEXC, OKX</t>
         </is>
       </c>
       <c r="BK36" s="24" t="n">
-        <v>1.6265</v>
+        <v>193.364</v>
       </c>
       <c r="BL36" s="66" t="n">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
       <c r="BM36" s="67" t="n">
-        <v>0.16248</v>
+        <v>0.19339</v>
       </c>
       <c r="BN36" s="66" t="n"/>
       <c r="BO36" s="68" t="n"/>
       <c r="BP36" s="66" t="n">
-        <v>0.1</v>
+        <v>0.001</v>
       </c>
       <c r="BQ36" s="69" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="BR36" s="70" t="n">
-        <v>0.0005360800000000001</v>
+        <v>0.00125</v>
       </c>
       <c r="BS36" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT36" s="25" t="n">
-        <v>260373.8032099999</v>
+        <v>128396.02003</v>
       </c>
       <c r="BU36" s="70" t="n">
-        <v>0.01230920728704936</v>
+        <v>0.005170898185010034</v>
       </c>
       <c r="BV36" s="22" t="inlineStr">
         <is>
@@ -31666,13 +31720,13 @@
         </is>
       </c>
       <c r="O37" s="8" t="n">
-        <v>0.4114</v>
+        <v>0.4174</v>
       </c>
       <c r="P37" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q37" s="43" t="n">
-        <v>4.114</v>
+        <v>4.173999999999999</v>
       </c>
       <c r="R37" s="42" t="n">
         <v>0.0001</v>
@@ -31687,16 +31741,16 @@
         <v>50</v>
       </c>
       <c r="V37" s="46" t="n">
-        <v>0.00254656975289</v>
+        <v>-0.00524370524632</v>
       </c>
       <c r="W37" s="47" t="n">
         <v>4</v>
       </c>
       <c r="X37" s="9" t="n">
-        <v>1691251.622</v>
+        <v>1611930.004999999</v>
       </c>
       <c r="Y37" s="46" t="n">
-        <v>0.02430724355857778</v>
+        <v>0.02395783421178461</v>
       </c>
       <c r="Z37" s="6" t="inlineStr">
         <is>
@@ -31738,7 +31792,7 @@
       </c>
       <c r="AL37" s="10" t="inlineStr"/>
       <c r="AM37" s="16" t="n">
-        <v>0</v>
+        <v>0.4183312244340553</v>
       </c>
       <c r="AN37" s="54" t="n">
         <v>0.1</v>
@@ -31765,18 +31819,20 @@
         <v>4</v>
       </c>
       <c r="AV37" s="17" t="n">
-        <v>1341747.58086</v>
-      </c>
-      <c r="AW37" s="58" t="n"/>
+        <v>1604516.4058</v>
+      </c>
+      <c r="AW37" s="58" t="n">
+        <v>0.02392344497607392</v>
+      </c>
       <c r="AX37" s="14" t="inlineStr"/>
       <c r="AY37" s="20" t="n">
-        <v>0.411718</v>
+        <v>0.417898</v>
       </c>
       <c r="AZ37" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA37" s="61" t="n">
-        <v>0.4115</v>
+        <v>0.4174</v>
       </c>
       <c r="BB37" s="60" t="n">
         <v>0.0001</v>
@@ -31791,16 +31847,16 @@
         <v>50</v>
       </c>
       <c r="BF37" s="64" t="n">
-        <v>-0.0017</v>
+        <v>-0.0056</v>
       </c>
       <c r="BG37" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH37" s="21" t="n">
-        <v>746807.0767000001</v>
+        <v>763771.6392000002</v>
       </c>
       <c r="BI37" s="64" t="n">
-        <v>0.04860267314703123</v>
+        <v>0.04791566842356923</v>
       </c>
       <c r="BJ37" s="18" t="inlineStr">
         <is>
@@ -31808,13 +31864,13 @@
         </is>
       </c>
       <c r="BK37" s="24" t="n">
-        <v>0.41191</v>
+        <v>0.4179</v>
       </c>
       <c r="BL37" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM37" s="67" t="n">
-        <v>0.41186</v>
+        <v>0.41774</v>
       </c>
       <c r="BN37" s="66" t="n"/>
       <c r="BO37" s="68" t="n"/>
@@ -31831,10 +31887,10 @@
         <v>1</v>
       </c>
       <c r="BT37" s="25" t="n">
-        <v>108394.54671</v>
+        <v>99384.14276999999</v>
       </c>
       <c r="BU37" s="70" t="n">
-        <v>0.05098819987374058</v>
+        <v>0.009575333939767438</v>
       </c>
       <c r="BV37" s="22" t="inlineStr">
         <is>
@@ -31866,13 +31922,13 @@
       <c r="M38" s="40" t="n"/>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="8" t="n">
-        <v>85.95</v>
+        <v>86.15000000000001</v>
       </c>
       <c r="P38" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q38" s="43" t="n">
-        <v>0.8595</v>
+        <v>0.8615</v>
       </c>
       <c r="R38" s="42" t="n">
         <v>0.01</v>
@@ -31887,16 +31943,16 @@
         <v>20</v>
       </c>
       <c r="V38" s="46" t="n">
-        <v>0.005</v>
+        <v>-0.00661361236355</v>
       </c>
       <c r="W38" s="47" t="n">
         <v>4</v>
       </c>
       <c r="X38" s="9" t="n">
-        <v>198654.5368</v>
+        <v>276734.7362</v>
       </c>
       <c r="Y38" s="46" t="n">
-        <v>0.01163467132054115</v>
+        <v>0.01160766105630309</v>
       </c>
       <c r="Z38" s="6" t="inlineStr">
         <is>
@@ -31950,13 +32006,13 @@
       <c r="AW38" s="58" t="n"/>
       <c r="AX38" s="14" t="inlineStr"/>
       <c r="AY38" s="20" t="n">
-        <v>86</v>
+        <v>86.20099999999999</v>
       </c>
       <c r="AZ38" s="60" t="n">
         <v>0.1</v>
       </c>
       <c r="BA38" s="61" t="n">
-        <v>8.593999999999999</v>
+        <v>8.613</v>
       </c>
       <c r="BB38" s="60" t="n">
         <v>0.01</v>
@@ -31971,16 +32027,16 @@
         <v>25</v>
       </c>
       <c r="BF38" s="64" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0024</v>
       </c>
       <c r="BG38" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH38" s="21" t="n">
-        <v>93287.274</v>
+        <v>112425.652</v>
       </c>
       <c r="BI38" s="64" t="n">
-        <v>0.05818012566906813</v>
+        <v>0.1044932079414878</v>
       </c>
       <c r="BJ38" s="18" t="inlineStr">
         <is>
@@ -32094,7 +32150,7 @@
       </c>
       <c r="AL39" s="10" t="inlineStr"/>
       <c r="AM39" s="16" t="n">
-        <v>0</v>
+        <v>4066.332212457461</v>
       </c>
       <c r="AN39" s="54" t="n">
         <v>0.001</v>
@@ -32115,24 +32171,26 @@
         <v>50</v>
       </c>
       <c r="AT39" s="58" t="n">
-        <v>0.0005</v>
+        <v>-0.0018</v>
       </c>
       <c r="AU39" s="59" t="n">
         <v>4</v>
       </c>
       <c r="AV39" s="17" t="n">
-        <v>135186.17812</v>
-      </c>
-      <c r="AW39" s="58" t="n"/>
+        <v>249017.7354100001</v>
+      </c>
+      <c r="AW39" s="58" t="n">
+        <v>0.0223943221780154</v>
+      </c>
       <c r="AX39" s="14" t="inlineStr"/>
       <c r="AY39" s="20" t="n">
-        <v>4061.31</v>
+        <v>4065.99</v>
       </c>
       <c r="AZ39" s="60" t="n">
         <v>0.001</v>
       </c>
       <c r="BA39" s="61" t="n">
-        <v>4.06</v>
+        <v>4.0641</v>
       </c>
       <c r="BB39" s="60" t="n">
         <v>0.1</v>
@@ -32147,16 +32205,16 @@
         <v>100</v>
       </c>
       <c r="BF39" s="64" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="BG39" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH39" s="21" t="n">
-        <v>745658.5917000002</v>
+        <v>624621.1668999998</v>
       </c>
       <c r="BI39" s="64" t="n">
-        <v>0.01970443349754143</v>
+        <v>0.02952683250904931</v>
       </c>
       <c r="BJ39" s="18" t="inlineStr">
         <is>
@@ -32164,13 +32222,13 @@
         </is>
       </c>
       <c r="BK39" s="24" t="n">
-        <v>4059.45</v>
+        <v>4066.5</v>
       </c>
       <c r="BL39" s="66" t="n">
         <v>0.001</v>
       </c>
       <c r="BM39" s="67" t="n">
-        <v>4.058</v>
+        <v>4.0648</v>
       </c>
       <c r="BN39" s="66" t="n"/>
       <c r="BO39" s="68" t="n"/>
@@ -32187,10 +32245,10 @@
         <v>1</v>
       </c>
       <c r="BT39" s="25" t="n">
-        <v>549898.8718</v>
+        <v>306232.3089999999</v>
       </c>
       <c r="BU39" s="70" t="n">
-        <v>0.002464268112368385</v>
+        <v>0.002460145640619687</v>
       </c>
       <c r="BV39" s="22" t="inlineStr">
         <is>
@@ -32246,13 +32304,13 @@
         </is>
       </c>
       <c r="O40" s="8" t="n">
-        <v>0.0553</v>
+        <v>0.05533</v>
       </c>
       <c r="P40" s="42" t="n">
         <v>10</v>
       </c>
       <c r="Q40" s="43" t="n">
-        <v>0.553</v>
+        <v>0.5533</v>
       </c>
       <c r="R40" s="42" t="n">
         <v>1e-05</v>
@@ -32273,10 +32331,10 @@
         <v>4</v>
       </c>
       <c r="X40" s="9" t="n">
-        <v>477053.4415000001</v>
+        <v>438437.6066000001</v>
       </c>
       <c r="Y40" s="46" t="n">
-        <v>0.01808318264013765</v>
+        <v>0.01807337791432518</v>
       </c>
       <c r="Z40" s="6" t="inlineStr">
         <is>
@@ -32296,7 +32354,7 @@
       <c r="AK40" s="52" t="n"/>
       <c r="AL40" s="10" t="inlineStr"/>
       <c r="AM40" s="16" t="n">
-        <v>0</v>
+        <v>0.0554340305455573</v>
       </c>
       <c r="AN40" s="54" t="n">
         <v>1</v>
@@ -32317,24 +32375,26 @@
         <v>75</v>
       </c>
       <c r="AT40" s="58" t="n">
-        <v>0.0035</v>
+        <v>0.005</v>
       </c>
       <c r="AU40" s="59" t="n">
         <v>4</v>
       </c>
       <c r="AV40" s="17" t="n">
-        <v>333763.1495999999</v>
-      </c>
-      <c r="AW40" s="58" t="n"/>
+        <v>665145.5237999998</v>
+      </c>
+      <c r="AW40" s="58" t="n">
+        <v>0.03609456776754951</v>
+      </c>
       <c r="AX40" s="14" t="inlineStr"/>
       <c r="AY40" s="20" t="n">
-        <v>0.05537</v>
+        <v>0.05542</v>
       </c>
       <c r="AZ40" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA40" s="61" t="n">
-        <v>0.5535</v>
+        <v>0.5539999999999999</v>
       </c>
       <c r="BB40" s="60" t="n">
         <v>1e-05</v>
@@ -32349,16 +32409,16 @@
         <v>75</v>
       </c>
       <c r="BF40" s="64" t="n">
-        <v>0.0024</v>
+        <v>0.0049</v>
       </c>
       <c r="BG40" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH40" s="21" t="n">
-        <v>285406.5826999999</v>
+        <v>287817.7517</v>
       </c>
       <c r="BI40" s="64" t="n">
-        <v>0.01806684733513301</v>
+        <v>0.0361010830324895</v>
       </c>
       <c r="BJ40" s="18" t="inlineStr">
         <is>
@@ -32366,13 +32426,13 @@
         </is>
       </c>
       <c r="BK40" s="24" t="n">
-        <v>0.055375</v>
+        <v>0.05545</v>
       </c>
       <c r="BL40" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM40" s="67" t="n">
-        <v>0.055355</v>
+        <v>0.055422</v>
       </c>
       <c r="BN40" s="66" t="n"/>
       <c r="BO40" s="68" t="n"/>
@@ -32389,10 +32449,10 @@
         <v>1</v>
       </c>
       <c r="BT40" s="25" t="n">
-        <v>99678.01232899999</v>
+        <v>164593.453235</v>
       </c>
       <c r="BU40" s="70" t="n">
-        <v>0.02167825851322938</v>
+        <v>0.01082602576593963</v>
       </c>
       <c r="BV40" s="22" t="inlineStr">
         <is>
@@ -32448,13 +32508,13 @@
         </is>
       </c>
       <c r="O41" s="8" t="n">
-        <v>0.5995</v>
+        <v>0.5989</v>
       </c>
       <c r="P41" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q41" s="43" t="n">
-        <v>0.5995</v>
+        <v>0.5989</v>
       </c>
       <c r="R41" s="42" t="n">
         <v>0.0001</v>
@@ -32469,16 +32529,16 @@
         <v>50</v>
       </c>
       <c r="V41" s="46" t="n">
-        <v>0.00486943123392</v>
+        <v>-0.00346845896069</v>
       </c>
       <c r="W41" s="47" t="n">
         <v>4</v>
       </c>
       <c r="X41" s="9" t="n">
-        <v>769130.588</v>
+        <v>761179.1446000002</v>
       </c>
       <c r="Y41" s="46" t="n">
-        <v>0.0166805671392809</v>
+        <v>0.01669727834362815</v>
       </c>
       <c r="Z41" s="6" t="inlineStr">
         <is>
@@ -32520,7 +32580,7 @@
       </c>
       <c r="AL41" s="10" t="inlineStr"/>
       <c r="AM41" s="16" t="n">
-        <v>0</v>
+        <v>0.5999134109359205</v>
       </c>
       <c r="AN41" s="54" t="n">
         <v>1</v>
@@ -32547,18 +32607,20 @@
         <v>4</v>
       </c>
       <c r="AV41" s="17" t="n">
-        <v>556291.3417</v>
-      </c>
-      <c r="AW41" s="58" t="n"/>
+        <v>1112123.8154</v>
+      </c>
+      <c r="AW41" s="58" t="n">
+        <v>0.01668891855809413</v>
+      </c>
       <c r="AX41" s="14" t="inlineStr"/>
       <c r="AY41" s="20" t="n">
-        <v>0.60039</v>
+        <v>0.5997400000000001</v>
       </c>
       <c r="AZ41" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA41" s="61" t="n">
-        <v>6</v>
+        <v>5.993</v>
       </c>
       <c r="BB41" s="60" t="n">
         <v>0.0001</v>
@@ -32573,16 +32635,16 @@
         <v>75</v>
       </c>
       <c r="BF41" s="64" t="n">
-        <v>0.0015</v>
+        <v>-0.0005</v>
       </c>
       <c r="BG41" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH41" s="21" t="n">
-        <v>395011.237</v>
+        <v>384052.8009999999</v>
       </c>
       <c r="BI41" s="64" t="n">
-        <v>0.03333333333332966</v>
+        <v>0.03337226764560137</v>
       </c>
       <c r="BJ41" s="18" t="inlineStr">
         <is>
@@ -32590,13 +32652,13 @@
         </is>
       </c>
       <c r="BK41" s="24" t="n">
-        <v>0.60055</v>
+        <v>0.59975</v>
       </c>
       <c r="BL41" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM41" s="67" t="n">
-        <v>0.6001</v>
+        <v>0.59943</v>
       </c>
       <c r="BN41" s="66" t="n"/>
       <c r="BO41" s="68" t="n"/>
@@ -32607,16 +32669,16 @@
         <v>5</v>
       </c>
       <c r="BR41" s="70" t="n">
-        <v>0.00027418</v>
+        <v>0.00125</v>
       </c>
       <c r="BS41" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT41" s="25" t="n">
-        <v>76300.22444999998</v>
+        <v>99040.99334</v>
       </c>
       <c r="BU41" s="70" t="n">
-        <v>0.001666388935169887</v>
+        <v>0.008341257527984001</v>
       </c>
       <c r="BV41" s="22" t="inlineStr">
         <is>
@@ -32632,7 +32694,7 @@
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>USDD</t>
+          <t>RLUSD</t>
         </is>
       </c>
       <c r="C42" s="4" t="n"/>
@@ -32716,7 +32778,7 @@
       </c>
       <c r="B43" s="35" t="inlineStr">
         <is>
-          <t>RLUSD</t>
+          <t>USDD</t>
         </is>
       </c>
       <c r="C43" s="4" t="n"/>
@@ -32840,13 +32902,13 @@
         </is>
       </c>
       <c r="O44" s="8" t="n">
-        <v>96.65000000000001</v>
+        <v>97.45999999999999</v>
       </c>
       <c r="P44" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q44" s="43" t="n">
-        <v>0.9665000000000002</v>
+        <v>0.9746000000000001</v>
       </c>
       <c r="R44" s="42" t="n">
         <v>0.01</v>
@@ -32861,16 +32923,16 @@
         <v>50</v>
       </c>
       <c r="V44" s="46" t="n">
-        <v>-0.00515021418056</v>
+        <v>-0.0006055908027800001</v>
       </c>
       <c r="W44" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X44" s="9" t="n">
-        <v>1040614.496499999</v>
+        <v>961299.8989000001</v>
       </c>
       <c r="Y44" s="46" t="n">
-        <v>0.01034661148474404</v>
+        <v>0.01026061974143763</v>
       </c>
       <c r="Z44" s="6" t="inlineStr">
         <is>
@@ -32912,7 +32974,7 @@
       </c>
       <c r="AL44" s="10" t="inlineStr"/>
       <c r="AM44" s="16" t="n">
-        <v>0</v>
+        <v>97.5546604654909</v>
       </c>
       <c r="AN44" s="54" t="n">
         <v>0.1</v>
@@ -32939,18 +33001,20 @@
         <v>8</v>
       </c>
       <c r="AV44" s="17" t="n">
-        <v>776237.9190000001</v>
-      </c>
-      <c r="AW44" s="58" t="n"/>
+        <v>1925286.13</v>
+      </c>
+      <c r="AW44" s="58" t="n">
+        <v>0.01025746230383128</v>
+      </c>
       <c r="AX44" s="14" t="inlineStr"/>
       <c r="AY44" s="20" t="n">
-        <v>96.812</v>
+        <v>97.502</v>
       </c>
       <c r="AZ44" s="60" t="n">
         <v>0.01</v>
       </c>
       <c r="BA44" s="61" t="n">
-        <v>0.9673999999999999</v>
+        <v>0.9749</v>
       </c>
       <c r="BB44" s="60" t="n">
         <v>0.01</v>
@@ -32965,16 +33029,16 @@
         <v>75</v>
       </c>
       <c r="BF44" s="64" t="n">
-        <v>-0.0128</v>
+        <v>-0.006399999999999999</v>
       </c>
       <c r="BG44" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH44" s="21" t="n">
-        <v>319981.5834000001</v>
+        <v>405170.2112999998</v>
       </c>
       <c r="BI44" s="64" t="n">
-        <v>0.02067397146992995</v>
+        <v>0.03077238691147927</v>
       </c>
       <c r="BJ44" s="18" t="inlineStr">
         <is>
@@ -32982,13 +33046,13 @@
         </is>
       </c>
       <c r="BK44" s="24" t="n">
-        <v>96.785</v>
+        <v>97.545</v>
       </c>
       <c r="BL44" s="66" t="n">
         <v>0.01</v>
       </c>
       <c r="BM44" s="67" t="n">
-        <v>0.9673999999999999</v>
+        <v>0.97516</v>
       </c>
       <c r="BN44" s="66" t="n"/>
       <c r="BO44" s="68" t="n"/>
@@ -33005,10 +33069,10 @@
         <v>1</v>
       </c>
       <c r="BT44" s="25" t="n">
-        <v>96705.40518</v>
+        <v>176991.76138</v>
       </c>
       <c r="BU44" s="70" t="n">
-        <v>0.001033698573486215</v>
+        <v>0.01128020017228956</v>
       </c>
       <c r="BV44" s="22" t="inlineStr">
         <is>
@@ -33064,13 +33128,13 @@
         </is>
       </c>
       <c r="O45" s="8" t="n">
-        <v>0.05673</v>
+        <v>0.05703</v>
       </c>
       <c r="P45" s="42" t="n">
         <v>100</v>
       </c>
       <c r="Q45" s="43" t="n">
-        <v>5.673</v>
+        <v>5.702999999999999</v>
       </c>
       <c r="R45" s="42" t="n">
         <v>1e-05</v>
@@ -33085,16 +33149,16 @@
         <v>20</v>
       </c>
       <c r="V45" s="46" t="n">
-        <v>-0.00263352307575</v>
+        <v>0.005</v>
       </c>
       <c r="W45" s="47" t="n">
         <v>4</v>
       </c>
       <c r="X45" s="9" t="n">
-        <v>56164.75400000002</v>
+        <v>52873.50599999998</v>
       </c>
       <c r="Y45" s="46" t="n">
-        <v>0.01762735765908007</v>
+        <v>0.03506926179203785</v>
       </c>
       <c r="Z45" s="6" t="inlineStr">
         <is>
@@ -33114,7 +33178,7 @@
       <c r="AK45" s="52" t="n"/>
       <c r="AL45" s="10" t="inlineStr"/>
       <c r="AM45" s="16" t="n">
-        <v>0</v>
+        <v>0.0571433402656062</v>
       </c>
       <c r="AN45" s="54" t="n">
         <v>1</v>
@@ -33141,18 +33205,20 @@
         <v>4</v>
       </c>
       <c r="AV45" s="17" t="n">
-        <v>184670.7813</v>
-      </c>
-      <c r="AW45" s="58" t="n"/>
+        <v>178772.9041200001</v>
+      </c>
+      <c r="AW45" s="58" t="n">
+        <v>0.05261311820413067</v>
+      </c>
       <c r="AX45" s="14" t="inlineStr"/>
       <c r="AY45" s="20" t="n">
-        <v>0.056869</v>
+        <v>0.057139</v>
       </c>
       <c r="AZ45" s="60" t="n">
         <v>100</v>
       </c>
       <c r="BA45" s="61" t="n">
-        <v>5.657</v>
+        <v>5.691</v>
       </c>
       <c r="BB45" s="60" t="n">
         <v>1e-05</v>
@@ -33167,16 +33233,16 @@
         <v>50</v>
       </c>
       <c r="BF45" s="64" t="n">
-        <v>0.0003</v>
+        <v>0.005</v>
       </c>
       <c r="BG45" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH45" s="21" t="n">
-        <v>12780.065</v>
+        <v>11554.041</v>
       </c>
       <c r="BI45" s="64" t="n">
-        <v>0.1237404984974379</v>
+        <v>0.07028641714988293</v>
       </c>
       <c r="BJ45" s="18" t="inlineStr">
         <is>
@@ -33184,13 +33250,13 @@
         </is>
       </c>
       <c r="BK45" s="24" t="n">
-        <v>0.05682</v>
+        <v>0.05714</v>
       </c>
       <c r="BL45" s="66" t="n">
         <v>1</v>
       </c>
       <c r="BM45" s="67" t="n">
-        <v>0.056785</v>
+        <v>0.057091</v>
       </c>
       <c r="BN45" s="66" t="n"/>
       <c r="BO45" s="68" t="n"/>
@@ -33207,10 +33273,10 @@
         <v>1</v>
       </c>
       <c r="BT45" s="25" t="n">
-        <v>26321.632766</v>
+        <v>24590.497042</v>
       </c>
       <c r="BU45" s="70" t="n">
-        <v>0.001761028440611077</v>
+        <v>0.02452225394545571</v>
       </c>
       <c r="BV45" s="22" t="inlineStr">
         <is>
@@ -33300,13 +33366,13 @@
       <c r="AW46" s="58" t="n"/>
       <c r="AX46" s="14" t="inlineStr"/>
       <c r="AY46" s="20" t="n">
-        <v>0.3958</v>
+        <v>0.3962</v>
       </c>
       <c r="AZ46" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA46" s="61" t="n">
-        <v>0.3958</v>
+        <v>0.3971</v>
       </c>
       <c r="BB46" s="60" t="n">
         <v>0.0001</v>
@@ -33321,16 +33387,16 @@
         <v>25</v>
       </c>
       <c r="BF46" s="64" t="n">
-        <v>0.0143</v>
+        <v>0.005</v>
       </c>
       <c r="BG46" s="65" t="n">
         <v>4</v>
       </c>
       <c r="BH46" s="21" t="n">
-        <v>43473.63029999999</v>
+        <v>36143.51690000001</v>
       </c>
       <c r="BI46" s="64" t="n">
-        <v>0.1010611419909074</v>
+        <v>0.07554772097708952</v>
       </c>
       <c r="BJ46" s="18" t="inlineStr">
         <is>
@@ -33338,13 +33404,13 @@
         </is>
       </c>
       <c r="BK46" s="24" t="n">
-        <v>0.39775</v>
+        <v>0.39795</v>
       </c>
       <c r="BL46" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM46" s="67" t="n">
-        <v>0.039731</v>
+        <v>0.03974900000000001</v>
       </c>
       <c r="BN46" s="66" t="n"/>
       <c r="BO46" s="68" t="n"/>
@@ -33355,16 +33421,16 @@
         <v>5</v>
       </c>
       <c r="BR46" s="70" t="n">
-        <v>-0.00289606</v>
+        <v>-0.00476434</v>
       </c>
       <c r="BS46" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT46" s="25" t="n">
-        <v>70574.93507799999</v>
+        <v>77020.63764800002</v>
       </c>
       <c r="BU46" s="70" t="n">
-        <v>0.03272004228436711</v>
+        <v>0.02264207904602241</v>
       </c>
       <c r="BV46" s="22" t="inlineStr">
         <is>
@@ -33420,13 +33486,13 @@
         </is>
       </c>
       <c r="O47" s="8" t="n">
-        <v>0.7678</v>
+        <v>0.769</v>
       </c>
       <c r="P47" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q47" s="43" t="n">
-        <v>0.7678</v>
+        <v>0.769</v>
       </c>
       <c r="R47" s="42" t="n">
         <v>0.0001</v>
@@ -33441,16 +33507,16 @@
         <v>50</v>
       </c>
       <c r="V47" s="46" t="n">
-        <v>-0.00251254096445</v>
+        <v>0.00011848736981</v>
       </c>
       <c r="W47" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X47" s="9" t="n">
-        <v>794633.4848000001</v>
+        <v>796870.7625</v>
       </c>
       <c r="Y47" s="46" t="n">
-        <v>0.01302422505860758</v>
+        <v>0.01300390117034967</v>
       </c>
       <c r="Z47" s="6" t="inlineStr">
         <is>
@@ -33492,7 +33558,7 @@
       </c>
       <c r="AL47" s="10" t="inlineStr"/>
       <c r="AM47" s="16" t="n">
-        <v>0</v>
+        <v>0.7695280402862003</v>
       </c>
       <c r="AN47" s="54" t="n">
         <v>1</v>
@@ -33513,24 +33579,26 @@
         <v>75</v>
       </c>
       <c r="AT47" s="58" t="n">
-        <v>0.0005</v>
+        <v>0.0007999999999999999</v>
       </c>
       <c r="AU47" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV47" s="17" t="n">
-        <v>3505509.853</v>
-      </c>
-      <c r="AW47" s="58" t="n"/>
+        <v>3011228.91</v>
+      </c>
+      <c r="AW47" s="58" t="n">
+        <v>0.1301405517959398</v>
+      </c>
       <c r="AX47" s="14" t="inlineStr"/>
       <c r="AY47" s="20" t="n">
-        <v>0.7685</v>
+        <v>0.7695</v>
       </c>
       <c r="AZ47" s="60" t="n">
         <v>1</v>
       </c>
       <c r="BA47" s="61" t="n">
-        <v>0.768</v>
+        <v>0.769</v>
       </c>
       <c r="BB47" s="60" t="n">
         <v>0.001</v>
@@ -33545,16 +33613,16 @@
         <v>75</v>
       </c>
       <c r="BF47" s="64" t="n">
-        <v>0.01</v>
+        <v>0.0057</v>
       </c>
       <c r="BG47" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH47" s="21" t="n">
-        <v>366657.245</v>
+        <v>329378.827</v>
       </c>
       <c r="BI47" s="64" t="n">
-        <v>0.1302083333333335</v>
+        <v>0.1300390117035112</v>
       </c>
       <c r="BJ47" s="18" t="inlineStr">
         <is>
@@ -33562,13 +33630,13 @@
         </is>
       </c>
       <c r="BK47" s="24" t="n">
-        <v>0.7684</v>
+        <v>0.76935</v>
       </c>
       <c r="BL47" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM47" s="67" t="n">
-        <v>0.076811</v>
+        <v>0.07689700000000001</v>
       </c>
       <c r="BN47" s="66" t="n"/>
       <c r="BO47" s="68" t="n"/>
@@ -33585,10 +33653,10 @@
         <v>1</v>
       </c>
       <c r="BT47" s="25" t="n">
-        <v>50180.69881300001</v>
+        <v>55192.18396499997</v>
       </c>
       <c r="BU47" s="70" t="n">
-        <v>0.02213224668341819</v>
+        <v>0.005201763397782616</v>
       </c>
       <c r="BV47" s="22" t="inlineStr">
         <is>
@@ -33690,7 +33758,7 @@
       </c>
       <c r="AL48" s="10" t="inlineStr"/>
       <c r="AM48" s="16" t="n">
-        <v>0</v>
+        <v>0.9592180529728792</v>
       </c>
       <c r="AN48" s="54" t="n">
         <v>1</v>
@@ -33717,18 +33785,20 @@
         <v>4</v>
       </c>
       <c r="AV48" s="17" t="n">
-        <v>14381.904</v>
-      </c>
-      <c r="AW48" s="58" t="n"/>
+        <v>22768.2741</v>
+      </c>
+      <c r="AW48" s="58" t="n">
+        <v>0.1145356101624313</v>
+      </c>
       <c r="AX48" s="14" t="inlineStr"/>
       <c r="AY48" s="20" t="n">
-        <v>0.958322</v>
+        <v>0.961396</v>
       </c>
       <c r="AZ48" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA48" s="61" t="n">
-        <v>9.574</v>
+        <v>9.613</v>
       </c>
       <c r="BB48" s="60" t="n">
         <v>0.0001</v>
@@ -33749,10 +33819,10 @@
         <v>8</v>
       </c>
       <c r="BH48" s="21" t="n">
-        <v>26225.129</v>
+        <v>28435.003</v>
       </c>
       <c r="BI48" s="64" t="n">
-        <v>0.1253394610403153</v>
+        <v>0.1664412774367975</v>
       </c>
       <c r="BJ48" s="18" t="inlineStr">
         <is>
@@ -33820,13 +33890,13 @@
         </is>
       </c>
       <c r="O49" s="8" t="n">
-        <v>3.9258</v>
+        <v>3.8365</v>
       </c>
       <c r="P49" s="42" t="n">
         <v>1</v>
       </c>
       <c r="Q49" s="43" t="n">
-        <v>3.9258</v>
+        <v>3.8365</v>
       </c>
       <c r="R49" s="42" t="n">
         <v>0.0001</v>
@@ -33841,16 +33911,16 @@
         <v>10</v>
       </c>
       <c r="V49" s="46" t="n">
-        <v>0.02557360640851</v>
+        <v>0.02373078968799</v>
       </c>
       <c r="W49" s="47" t="n">
         <v>4</v>
       </c>
       <c r="X49" s="9" t="n">
-        <v>26619.8039</v>
+        <v>14535.6643</v>
       </c>
       <c r="Y49" s="46" t="n">
-        <v>0.007641754546848769</v>
+        <v>0.0130327121073939</v>
       </c>
       <c r="Z49" s="6" t="inlineStr">
         <is>
@@ -33892,7 +33962,7 @@
       </c>
       <c r="AL49" s="10" t="inlineStr"/>
       <c r="AM49" s="16" t="n">
-        <v>0</v>
+        <v>3.825077016768987</v>
       </c>
       <c r="AN49" s="54" t="n">
         <v>1</v>
@@ -33919,18 +33989,20 @@
         <v>4</v>
       </c>
       <c r="AV49" s="17" t="n">
-        <v>12610.9005</v>
-      </c>
-      <c r="AW49" s="58" t="n"/>
+        <v>26875.4699</v>
+      </c>
+      <c r="AW49" s="58" t="n">
+        <v>0.03130952070341712</v>
+      </c>
       <c r="AX49" s="14" t="inlineStr"/>
       <c r="AY49" s="20" t="n">
-        <v>3.92705</v>
+        <v>3.82782</v>
       </c>
       <c r="AZ49" s="60" t="n">
         <v>10</v>
       </c>
       <c r="BA49" s="61" t="n">
-        <v>39.274</v>
+        <v>38.339</v>
       </c>
       <c r="BB49" s="60" t="n">
         <v>0.0001</v>
@@ -33951,10 +34023,10 @@
         <v>8</v>
       </c>
       <c r="BH49" s="21" t="n">
-        <v>27767.56299999999</v>
+        <v>42178.16799999999</v>
       </c>
       <c r="BI49" s="64" t="n">
-        <v>0.07384019962315788</v>
+        <v>0.04173296121442457</v>
       </c>
       <c r="BJ49" s="18" t="inlineStr">
         <is>
@@ -34022,13 +34094,13 @@
         </is>
       </c>
       <c r="O50" s="8" t="n">
-        <v>2.073</v>
+        <v>2.075</v>
       </c>
       <c r="P50" s="42" t="n">
         <v>0.01</v>
       </c>
       <c r="Q50" s="43" t="n">
-        <v>0.02073</v>
+        <v>0.02075</v>
       </c>
       <c r="R50" s="42" t="n">
         <v>0.001</v>
@@ -34043,16 +34115,16 @@
         <v>50</v>
       </c>
       <c r="V50" s="46" t="n">
-        <v>0.01</v>
+        <v>0.00183636207585</v>
       </c>
       <c r="W50" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X50" s="9" t="n">
-        <v>363112.30986</v>
+        <v>353401.5152099999</v>
       </c>
       <c r="Y50" s="46" t="n">
-        <v>0.04823926676313989</v>
+        <v>0.04819277108433204</v>
       </c>
       <c r="Z50" s="6" t="inlineStr">
         <is>
@@ -34094,7 +34166,7 @@
       </c>
       <c r="AL50" s="10" t="inlineStr"/>
       <c r="AM50" s="16" t="n">
-        <v>0</v>
+        <v>2.077521471843109</v>
       </c>
       <c r="AN50" s="54" t="n">
         <v>0.01</v>
@@ -34115,24 +34187,26 @@
         <v>50</v>
       </c>
       <c r="AT50" s="58" t="n">
-        <v>-0.0113</v>
+        <v>-0.0089</v>
       </c>
       <c r="AU50" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV50" s="17" t="n">
-        <v>499543.4297600003</v>
-      </c>
-      <c r="AW50" s="58" t="n"/>
+        <v>640484.8555399999</v>
+      </c>
+      <c r="AW50" s="58" t="n">
+        <v>0.04814636494946239</v>
+      </c>
       <c r="AX50" s="14" t="inlineStr"/>
       <c r="AY50" s="20" t="n">
-        <v>2.076</v>
+        <v>2.0785</v>
       </c>
       <c r="AZ50" s="60" t="n">
         <v>0.001</v>
       </c>
       <c r="BA50" s="61" t="n">
-        <v>0.002076</v>
+        <v>0.002077</v>
       </c>
       <c r="BB50" s="60" t="n">
         <v>0.001</v>
@@ -34153,10 +34227,10 @@
         <v>8</v>
       </c>
       <c r="BH50" s="21" t="n">
-        <v>249458.227761</v>
+        <v>223705.094749</v>
       </c>
       <c r="BI50" s="64" t="n">
-        <v>0.04816955684007176</v>
+        <v>0.0962927298989034</v>
       </c>
       <c r="BJ50" s="18" t="inlineStr">
         <is>
@@ -34164,13 +34238,13 @@
         </is>
       </c>
       <c r="BK50" s="24" t="n">
-        <v>2.079</v>
+        <v>2.07743</v>
       </c>
       <c r="BL50" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="BM50" s="67" t="n">
-        <v>0.20765</v>
+        <v>0.20748</v>
       </c>
       <c r="BN50" s="66" t="n"/>
       <c r="BO50" s="68" t="n"/>
@@ -34181,16 +34255,16 @@
         <v>5</v>
       </c>
       <c r="BR50" s="70" t="n">
-        <v>-0.00176546</v>
+        <v>-0.00318214</v>
       </c>
       <c r="BS50" s="71" t="n">
         <v>1</v>
       </c>
       <c r="BT50" s="25" t="n">
-        <v>75033.83164999999</v>
+        <v>96507.24424999999</v>
       </c>
       <c r="BU50" s="70" t="n">
-        <v>0.01926318324104985</v>
+        <v>0.01445922498554988</v>
       </c>
       <c r="BV50" s="22" t="inlineStr">
         <is>
@@ -34246,7 +34320,7 @@
       <c r="AK51" s="52" t="n"/>
       <c r="AL51" s="10" t="inlineStr"/>
       <c r="AM51" s="16" t="n">
-        <v>0</v>
+        <v>1.636015292798927</v>
       </c>
       <c r="AN51" s="54" t="n">
         <v>1</v>
@@ -34273,9 +34347,11 @@
         <v>8</v>
       </c>
       <c r="AV51" s="17" t="n">
-        <v>12007.3063</v>
-      </c>
-      <c r="AW51" s="58" t="n"/>
+        <v>29350.0806</v>
+      </c>
+      <c r="AW51" s="58" t="n">
+        <v>0.01223915305062114</v>
+      </c>
       <c r="AX51" s="14" t="inlineStr"/>
       <c r="AY51" s="20" t="n"/>
       <c r="AZ51" s="60" t="n"/>
@@ -34326,13 +34402,13 @@
       <c r="M52" s="40" t="n"/>
       <c r="N52" s="2" t="inlineStr"/>
       <c r="O52" s="8" t="n">
-        <v>2.735e-06</v>
+        <v>2.753e-06</v>
       </c>
       <c r="P52" s="42" t="n">
         <v>1000000</v>
       </c>
       <c r="Q52" s="43" t="n">
-        <v>2.735</v>
+        <v>2.753</v>
       </c>
       <c r="R52" s="42" t="n">
         <v>1e-09</v>
@@ -34347,16 +34423,16 @@
         <v>50</v>
       </c>
       <c r="V52" s="46" t="n">
-        <v>-0.00271477962072</v>
+        <v>0.00013191061197</v>
       </c>
       <c r="W52" s="47" t="n">
         <v>8</v>
       </c>
       <c r="X52" s="9" t="n">
-        <v>3021766.826000001</v>
+        <v>3744750.686</v>
       </c>
       <c r="Y52" s="46" t="n">
-        <v>0.03656307129799177</v>
+        <v>0.03632401017071019</v>
       </c>
       <c r="Z52" s="6" t="inlineStr">
         <is>
@@ -34376,7 +34452,7 @@
       <c r="AK52" s="52" t="n"/>
       <c r="AL52" s="10" t="inlineStr"/>
       <c r="AM52" s="16" t="n">
-        <v>0</v>
+        <v>2.7536316993e-06</v>
       </c>
       <c r="AN52" s="54" t="n">
         <v>1000</v>
@@ -34397,24 +34473,26 @@
         <v>75</v>
       </c>
       <c r="AT52" s="58" t="n">
-        <v>-0.009299999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="AU52" s="59" t="n">
         <v>8</v>
       </c>
       <c r="AV52" s="17" t="n">
-        <v>435420.6854149</v>
-      </c>
-      <c r="AW52" s="58" t="n"/>
+        <v>1450878.045626601</v>
+      </c>
+      <c r="AW52" s="58" t="n">
+        <v>0.01452538310696516</v>
+      </c>
       <c r="AX52" s="14" t="inlineStr"/>
       <c r="AY52" s="20" t="n">
-        <v>2.74083e-06</v>
+        <v>2.75667e-06</v>
       </c>
       <c r="AZ52" s="60" t="n">
         <v>10000000</v>
       </c>
       <c r="BA52" s="61" t="n">
-        <v>27.39</v>
+        <v>27.55</v>
       </c>
       <c r="BB52" s="60" t="n">
         <v>1e-09</v>
@@ -34429,16 +34507,16 @@
         <v>75</v>
       </c>
       <c r="BF52" s="64" t="n">
-        <v>-0.011</v>
+        <v>0.0026</v>
       </c>
       <c r="BG52" s="65" t="n">
         <v>8</v>
       </c>
       <c r="BH52" s="21" t="n">
-        <v>1531155.16</v>
+        <v>1225455.47</v>
       </c>
       <c r="BI52" s="64" t="n">
-        <v>0.03650967506389467</v>
+        <v>0.03629764065334488</v>
       </c>
       <c r="BJ52" s="18" t="inlineStr">
         <is>

</xml_diff>